<commit_message>
updated database (issues 13 & 14)
</commit_message>
<xml_diff>
--- a/FOSS4Spec.xlsx
+++ b/FOSS4Spec.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bryanh/Documents/Professional/Research/R_Pkgs/FOSS4Spectroscopy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA988ED5-D921-564C-8A49-DDFAB74C241D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D87021-F023-DE48-BE63-6DFCFA9CE71B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="17380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="glob" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4062" uniqueCount="1698">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4052" uniqueCount="1696">
   <si>
     <t>name</t>
   </si>
@@ -3928,15 +3928,6 @@
     <t>MIR, NIR</t>
   </si>
   <si>
-    <t>SimulatedLIBS</t>
-  </si>
-  <si>
-    <t>https://github.com/MKastek/SimulatedLIBS</t>
-  </si>
-  <si>
-    <t>SimulatedLIBS provides Python class to simulate LIBS spectra with NIST LIBS Database interface.</t>
-  </si>
-  <si>
     <t>simulateIRAS</t>
   </si>
   <si>
@@ -5114,6 +5105,9 @@
   </si>
   <si>
     <t>Tool to identify anomalous peaks in XRF spectra</t>
+  </si>
+  <si>
+    <t>https://github.com/Bluejee/OpenLIBS</t>
   </si>
 </sst>
 </file>
@@ -5468,7 +5462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J407"/>
+  <dimension ref="A1:J406"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.1640625" customWidth="1"/>
@@ -5514,7 +5508,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>1624</v>
+        <v>1621</v>
       </c>
       <c r="C2" t="s">
         <v>20</v>
@@ -5552,7 +5546,7 @@
         <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>14</v>
@@ -5610,7 +5604,7 @@
         <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>1645</v>
+        <v>1642</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
@@ -5817,7 +5811,7 @@
         <v>55</v>
       </c>
       <c r="G11" t="s">
-        <v>1644</v>
+        <v>1641</v>
       </c>
       <c r="H11" t="s">
         <v>10</v>
@@ -5840,7 +5834,7 @@
         <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>60</v>
@@ -5962,7 +5956,7 @@
         <v>81</v>
       </c>
       <c r="B16" t="s">
-        <v>1646</v>
+        <v>1643</v>
       </c>
       <c r="C16" t="s">
         <v>20</v>
@@ -6026,7 +6020,7 @@
         <v>90</v>
       </c>
       <c r="B18" t="s">
-        <v>1647</v>
+        <v>1644</v>
       </c>
       <c r="C18" t="s">
         <v>20</v>
@@ -6393,7 +6387,7 @@
         <v>10</v>
       </c>
       <c r="G29" t="s">
-        <v>1648</v>
+        <v>1645</v>
       </c>
       <c r="H29" t="s">
         <v>10</v>
@@ -6538,13 +6532,13 @@
         <v>163</v>
       </c>
       <c r="B34" t="s">
-        <v>1626</v>
+        <v>1623</v>
       </c>
       <c r="C34" t="s">
         <v>20</v>
       </c>
       <c r="D34" t="s">
-        <v>1666</v>
+        <v>1663</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>164</v>
@@ -6666,7 +6660,7 @@
         <v>180</v>
       </c>
       <c r="B38" t="s">
-        <v>1649</v>
+        <v>1646</v>
       </c>
       <c r="C38" t="s">
         <v>20</v>
@@ -6992,7 +6986,7 @@
         <v>20</v>
       </c>
       <c r="D48" t="s">
-        <v>1650</v>
+        <v>1647</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>223</v>
@@ -7111,22 +7105,22 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
+        <v>1624</v>
+      </c>
+      <c r="B52" t="s">
+        <v>1626</v>
+      </c>
+      <c r="C52" t="s">
+        <v>20</v>
+      </c>
+      <c r="D52" t="s">
+        <v>1622</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>1625</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>1627</v>
-      </c>
-      <c r="B52" t="s">
-        <v>1629</v>
-      </c>
-      <c r="C52" t="s">
-        <v>20</v>
-      </c>
-      <c r="D52" t="s">
-        <v>1625</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>1628</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>1630</v>
       </c>
       <c r="G52" t="s">
         <v>10</v>
@@ -7143,7 +7137,7 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>1651</v>
+        <v>1648</v>
       </c>
       <c r="B53" t="s">
         <v>243</v>
@@ -7178,7 +7172,7 @@
         <v>244</v>
       </c>
       <c r="B54" t="s">
-        <v>1652</v>
+        <v>1649</v>
       </c>
       <c r="C54" t="s">
         <v>20</v>
@@ -7280,7 +7274,7 @@
         <v>36</v>
       </c>
       <c r="D57" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>256</v>
@@ -7306,7 +7300,7 @@
         <v>261</v>
       </c>
       <c r="B58" t="s">
-        <v>1653</v>
+        <v>1650</v>
       </c>
       <c r="C58" t="s">
         <v>20</v>
@@ -7624,13 +7618,13 @@
         <v>301</v>
       </c>
       <c r="B68" t="s">
-        <v>1654</v>
+        <v>1651</v>
       </c>
       <c r="C68" t="s">
         <v>20</v>
       </c>
       <c r="D68" t="s">
-        <v>1655</v>
+        <v>1652</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>300</v>
@@ -7688,7 +7682,7 @@
         <v>309</v>
       </c>
       <c r="B70" t="s">
-        <v>1656</v>
+        <v>1653</v>
       </c>
       <c r="C70" t="s">
         <v>20</v>
@@ -7700,7 +7694,7 @@
         <v>310</v>
       </c>
       <c r="F70" t="s">
-        <v>1609</v>
+        <v>1606</v>
       </c>
       <c r="G70" t="s">
         <v>10</v>
@@ -7720,7 +7714,7 @@
         <v>312</v>
       </c>
       <c r="B71" t="s">
-        <v>1657</v>
+        <v>1654</v>
       </c>
       <c r="C71" t="s">
         <v>20</v>
@@ -8023,7 +8017,7 @@
         <v>10</v>
       </c>
       <c r="G80" t="s">
-        <v>1658</v>
+        <v>1655</v>
       </c>
       <c r="H80" t="s">
         <v>10</v>
@@ -8238,7 +8232,7 @@
         <v>20</v>
       </c>
       <c r="D87" t="s">
-        <v>1659</v>
+        <v>1656</v>
       </c>
       <c r="E87" s="1" t="s">
         <v>376</v>
@@ -8270,7 +8264,7 @@
         <v>20</v>
       </c>
       <c r="D88" t="s">
-        <v>1659</v>
+        <v>1656</v>
       </c>
       <c r="E88" s="1" t="s">
         <v>379</v>
@@ -8296,7 +8290,7 @@
         <v>381</v>
       </c>
       <c r="B89" t="s">
-        <v>1660</v>
+        <v>1657</v>
       </c>
       <c r="C89" t="s">
         <v>20</v>
@@ -8392,7 +8386,7 @@
         <v>393</v>
       </c>
       <c r="B92" t="s">
-        <v>1610</v>
+        <v>1607</v>
       </c>
       <c r="C92" t="s">
         <v>20</v>
@@ -8613,22 +8607,22 @@
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>1634</v>
+        <v>1631</v>
       </c>
       <c r="B99" t="s">
-        <v>1692</v>
+        <v>1689</v>
       </c>
       <c r="C99" t="s">
         <v>20</v>
       </c>
       <c r="D99" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>1635</v>
+        <v>1632</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>1636</v>
+        <v>1633</v>
       </c>
       <c r="G99" t="s">
         <v>10</v>
@@ -8645,19 +8639,19 @@
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>1631</v>
+        <v>1628</v>
       </c>
       <c r="B100" t="s">
-        <v>1633</v>
+        <v>1630</v>
       </c>
       <c r="C100" t="s">
         <v>20</v>
       </c>
       <c r="D100" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>1632</v>
+        <v>1629</v>
       </c>
       <c r="F100" t="s">
         <v>10</v>
@@ -8680,7 +8674,7 @@
         <v>423</v>
       </c>
       <c r="B101" t="s">
-        <v>1611</v>
+        <v>1608</v>
       </c>
       <c r="C101" t="s">
         <v>20</v>
@@ -8750,7 +8744,7 @@
         <v>20</v>
       </c>
       <c r="D103" t="s">
-        <v>1688</v>
+        <v>1685</v>
       </c>
       <c r="E103" s="1" t="s">
         <v>431</v>
@@ -9192,7 +9186,7 @@
         <v>481</v>
       </c>
       <c r="B117" t="s">
-        <v>1612</v>
+        <v>1609</v>
       </c>
       <c r="C117" t="s">
         <v>20</v>
@@ -9230,7 +9224,7 @@
         <v>20</v>
       </c>
       <c r="D118" t="s">
-        <v>1689</v>
+        <v>1686</v>
       </c>
       <c r="E118" s="1" t="s">
         <v>484</v>
@@ -9326,7 +9320,7 @@
         <v>20</v>
       </c>
       <c r="D121" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E121" s="1" t="s">
         <v>496</v>
@@ -9390,7 +9384,7 @@
         <v>36</v>
       </c>
       <c r="D123" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E123" s="1" t="s">
         <v>505</v>
@@ -9704,7 +9698,7 @@
         <v>547</v>
       </c>
       <c r="B133" t="s">
-        <v>1661</v>
+        <v>1658</v>
       </c>
       <c r="C133" t="s">
         <v>20</v>
@@ -9902,7 +9896,7 @@
         <v>47</v>
       </c>
       <c r="D139" t="s">
-        <v>1671</v>
+        <v>1668</v>
       </c>
       <c r="E139" s="1" t="s">
         <v>568</v>
@@ -9928,13 +9922,13 @@
         <v>571</v>
       </c>
       <c r="B140" t="s">
-        <v>1662</v>
+        <v>1659</v>
       </c>
       <c r="C140" t="s">
         <v>20</v>
       </c>
       <c r="D140" t="s">
-        <v>1663</v>
+        <v>1660</v>
       </c>
       <c r="E140" s="1" t="s">
         <v>572</v>
@@ -10231,7 +10225,7 @@
         <v>10</v>
       </c>
       <c r="G149" t="s">
-        <v>1613</v>
+        <v>1610</v>
       </c>
       <c r="H149" t="s">
         <v>10</v>
@@ -10248,7 +10242,7 @@
         <v>611</v>
       </c>
       <c r="B150" t="s">
-        <v>1691</v>
+        <v>1688</v>
       </c>
       <c r="C150" t="s">
         <v>20</v>
@@ -10862,7 +10856,7 @@
         <v>20</v>
       </c>
       <c r="D169" t="s">
-        <v>1664</v>
+        <v>1661</v>
       </c>
       <c r="E169" s="1" t="s">
         <v>691</v>
@@ -10920,7 +10914,7 @@
         <v>698</v>
       </c>
       <c r="B171" t="s">
-        <v>1665</v>
+        <v>1662</v>
       </c>
       <c r="C171" t="s">
         <v>20</v>
@@ -12040,7 +12034,7 @@
         <v>850</v>
       </c>
       <c r="B206" t="s">
-        <v>1681</v>
+        <v>1678</v>
       </c>
       <c r="C206" t="s">
         <v>20</v>
@@ -12264,7 +12258,7 @@
         <v>878</v>
       </c>
       <c r="B213" t="s">
-        <v>1690</v>
+        <v>1687</v>
       </c>
       <c r="C213" t="s">
         <v>229</v>
@@ -12325,19 +12319,19 @@
     </row>
     <row r="215" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
-        <v>1637</v>
+        <v>1634</v>
       </c>
       <c r="B215" t="s">
-        <v>1614</v>
+        <v>1611</v>
       </c>
       <c r="C215" t="s">
         <v>20</v>
       </c>
       <c r="D215" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E215" s="1" t="s">
-        <v>1638</v>
+        <v>1635</v>
       </c>
       <c r="F215" t="s">
         <v>10</v>
@@ -12349,7 +12343,7 @@
         <v>10</v>
       </c>
       <c r="I215" t="s">
-        <v>1637</v>
+        <v>1634</v>
       </c>
       <c r="J215" t="s">
         <v>10</v>
@@ -12369,7 +12363,7 @@
         <v>89</v>
       </c>
       <c r="E216" s="1" t="s">
-        <v>879</v>
+        <v>1695</v>
       </c>
       <c r="F216" s="1" t="s">
         <v>879</v>
@@ -12398,7 +12392,7 @@
         <v>36</v>
       </c>
       <c r="D217" t="s">
-        <v>1666</v>
+        <v>1663</v>
       </c>
       <c r="E217" s="1" t="s">
         <v>887</v>
@@ -12424,13 +12418,13 @@
         <v>891</v>
       </c>
       <c r="B218" t="s">
-        <v>1693</v>
+        <v>1690</v>
       </c>
       <c r="C218" t="s">
         <v>20</v>
       </c>
       <c r="D218" t="s">
-        <v>1666</v>
+        <v>1663</v>
       </c>
       <c r="E218" s="1" t="s">
         <v>892</v>
@@ -12462,7 +12456,7 @@
         <v>20</v>
       </c>
       <c r="D219" t="s">
-        <v>1666</v>
+        <v>1663</v>
       </c>
       <c r="E219" s="1" t="s">
         <v>895</v>
@@ -12744,7 +12738,7 @@
         <v>933</v>
       </c>
       <c r="B228" t="s">
-        <v>1667</v>
+        <v>1664</v>
       </c>
       <c r="C228" t="s">
         <v>20</v>
@@ -13061,7 +13055,7 @@
     </row>
     <row r="238" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
-        <v>1687</v>
+        <v>1684</v>
       </c>
       <c r="B238" t="s">
         <v>975</v>
@@ -13093,19 +13087,19 @@
     </row>
     <row r="239" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="B239" t="s">
-        <v>1641</v>
+        <v>1638</v>
       </c>
       <c r="C239" t="s">
         <v>36</v>
       </c>
       <c r="D239" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E239" s="1" t="s">
-        <v>1640</v>
+        <v>1637</v>
       </c>
       <c r="F239" t="s">
         <v>10</v>
@@ -13256,13 +13250,13 @@
         <v>995</v>
       </c>
       <c r="B244" t="s">
-        <v>1642</v>
+        <v>1639</v>
       </c>
       <c r="C244" t="s">
         <v>20</v>
       </c>
       <c r="D244" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E244" s="1" t="s">
         <v>996</v>
@@ -13416,7 +13410,7 @@
         <v>1013</v>
       </c>
       <c r="B249" t="s">
-        <v>1615</v>
+        <v>1612</v>
       </c>
       <c r="C249" t="s">
         <v>20</v>
@@ -13733,7 +13727,7 @@
     </row>
     <row r="259" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
-        <v>1606</v>
+        <v>1603</v>
       </c>
       <c r="B259" t="s">
         <v>1052</v>
@@ -13748,10 +13742,10 @@
         <v>1051</v>
       </c>
       <c r="F259" t="s">
-        <v>1608</v>
+        <v>1605</v>
       </c>
       <c r="G259" t="s">
-        <v>1607</v>
+        <v>1604</v>
       </c>
     </row>
     <row r="260" spans="1:10" x14ac:dyDescent="0.2">
@@ -13765,7 +13759,7 @@
         <v>20</v>
       </c>
       <c r="D260" t="s">
-        <v>1668</v>
+        <v>1665</v>
       </c>
       <c r="E260" s="1" t="s">
         <v>1054</v>
@@ -13855,7 +13849,7 @@
         <v>1065</v>
       </c>
       <c r="B263" t="s">
-        <v>1616</v>
+        <v>1613</v>
       </c>
       <c r="C263" t="s">
         <v>20</v>
@@ -13887,13 +13881,13 @@
         <v>1067</v>
       </c>
       <c r="B264" t="s">
-        <v>1643</v>
+        <v>1640</v>
       </c>
       <c r="C264" t="s">
         <v>20</v>
       </c>
       <c r="D264" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E264" s="1" t="s">
         <v>1068</v>
@@ -14172,10 +14166,10 @@
     </row>
     <row r="273" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
-        <v>1617</v>
+        <v>1614</v>
       </c>
       <c r="B273" t="s">
-        <v>1619</v>
+        <v>1616</v>
       </c>
       <c r="C273" t="s">
         <v>20</v>
@@ -14184,7 +14178,7 @@
         <v>70</v>
       </c>
       <c r="E273" s="1" t="s">
-        <v>1618</v>
+        <v>1615</v>
       </c>
       <c r="F273" t="s">
         <v>10</v>
@@ -14207,7 +14201,7 @@
         <v>1104</v>
       </c>
       <c r="B274" t="s">
-        <v>1669</v>
+        <v>1666</v>
       </c>
       <c r="C274" t="s">
         <v>20</v>
@@ -14303,7 +14297,7 @@
         <v>1117</v>
       </c>
       <c r="B277" t="s">
-        <v>1694</v>
+        <v>1691</v>
       </c>
       <c r="C277" t="s">
         <v>20</v>
@@ -14469,7 +14463,7 @@
         <v>20</v>
       </c>
       <c r="D282" t="s">
-        <v>1670</v>
+        <v>1667</v>
       </c>
       <c r="E282" s="1" t="s">
         <v>1137</v>
@@ -14501,7 +14495,7 @@
         <v>20</v>
       </c>
       <c r="D283" t="s">
-        <v>1670</v>
+        <v>1667</v>
       </c>
       <c r="E283" s="1" t="s">
         <v>1141</v>
@@ -14533,7 +14527,7 @@
         <v>20</v>
       </c>
       <c r="D284" t="s">
-        <v>1670</v>
+        <v>1667</v>
       </c>
       <c r="E284" s="1" t="s">
         <v>1144</v>
@@ -14597,7 +14591,7 @@
         <v>20</v>
       </c>
       <c r="D286" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E286" s="1" t="s">
         <v>1151</v>
@@ -14629,7 +14623,7 @@
         <v>20</v>
       </c>
       <c r="D287" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="E287" s="1" t="s">
         <v>1154</v>
@@ -14975,7 +14969,7 @@
         <v>1192</v>
       </c>
       <c r="B298" t="s">
-        <v>1695</v>
+        <v>1692</v>
       </c>
       <c r="C298" t="s">
         <v>20</v>
@@ -15647,7 +15641,7 @@
         <v>1274</v>
       </c>
       <c r="B319" t="s">
-        <v>1672</v>
+        <v>1669</v>
       </c>
       <c r="C319" t="s">
         <v>20</v>
@@ -15711,7 +15705,7 @@
         <v>1280</v>
       </c>
       <c r="B321" t="s">
-        <v>1696</v>
+        <v>1693</v>
       </c>
       <c r="C321" t="s">
         <v>20</v>
@@ -15813,7 +15807,7 @@
         <v>20</v>
       </c>
       <c r="D324" t="s">
-        <v>1673</v>
+        <v>1670</v>
       </c>
       <c r="E324" s="1" t="s">
         <v>1294</v>
@@ -15877,19 +15871,19 @@
         <v>20</v>
       </c>
       <c r="D326" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="E326" s="1" t="s">
         <v>1303</v>
       </c>
       <c r="F326" s="1" t="s">
-        <v>1303</v>
+        <v>1305</v>
       </c>
       <c r="G326" t="s">
         <v>10</v>
       </c>
       <c r="H326" t="s">
-        <v>10</v>
+        <v>1306</v>
       </c>
       <c r="I326" t="s">
         <v>10</v>
@@ -15900,31 +15894,31 @@
     </row>
     <row r="327" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A327" t="s">
-        <v>1305</v>
+        <v>1307</v>
       </c>
       <c r="B327" t="s">
-        <v>1307</v>
+        <v>1309</v>
       </c>
       <c r="C327" t="s">
         <v>20</v>
       </c>
       <c r="D327" t="s">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="E327" s="1" t="s">
-        <v>1306</v>
-      </c>
-      <c r="F327" s="1" t="s">
         <v>1308</v>
       </c>
+      <c r="F327" t="s">
+        <v>10</v>
+      </c>
       <c r="G327" t="s">
         <v>10</v>
       </c>
       <c r="H327" t="s">
-        <v>1309</v>
+        <v>10</v>
       </c>
       <c r="I327" t="s">
-        <v>10</v>
+        <v>1310</v>
       </c>
       <c r="J327" t="s">
         <v>10</v>
@@ -15932,31 +15926,31 @@
     </row>
     <row r="328" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A328" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="B328" t="s">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="C328" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="D328" t="s">
         <v>31</v>
       </c>
       <c r="E328" s="1" t="s">
-        <v>1311</v>
-      </c>
-      <c r="F328" t="s">
-        <v>10</v>
-      </c>
-      <c r="G328" t="s">
-        <v>10</v>
+        <v>1312</v>
+      </c>
+      <c r="F328" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="G328" s="1" t="s">
+        <v>1314</v>
       </c>
       <c r="H328" t="s">
         <v>10</v>
       </c>
       <c r="I328" t="s">
-        <v>1313</v>
+        <v>10</v>
       </c>
       <c r="J328" t="s">
         <v>10</v>
@@ -15964,25 +15958,25 @@
     </row>
     <row r="329" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A329" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="B329" t="s">
+        <v>1317</v>
+      </c>
+      <c r="C329" t="s">
+        <v>20</v>
+      </c>
+      <c r="D329" t="s">
+        <v>161</v>
+      </c>
+      <c r="E329" s="1" t="s">
         <v>1316</v>
       </c>
-      <c r="C329" t="s">
-        <v>36</v>
-      </c>
-      <c r="D329" t="s">
-        <v>31</v>
-      </c>
-      <c r="E329" s="1" t="s">
-        <v>1315</v>
-      </c>
-      <c r="F329" s="1" t="s">
-        <v>1315</v>
-      </c>
-      <c r="G329" s="1" t="s">
-        <v>1317</v>
+      <c r="F329" t="s">
+        <v>10</v>
+      </c>
+      <c r="G329" t="s">
+        <v>10</v>
       </c>
       <c r="H329" t="s">
         <v>10</v>
@@ -16010,14 +16004,14 @@
       <c r="E330" s="1" t="s">
         <v>1319</v>
       </c>
-      <c r="F330" t="s">
-        <v>10</v>
+      <c r="F330" s="1" t="s">
+        <v>1321</v>
       </c>
       <c r="G330" t="s">
         <v>10</v>
       </c>
       <c r="H330" t="s">
-        <v>10</v>
+        <v>909</v>
       </c>
       <c r="I330" t="s">
         <v>10</v>
@@ -16028,28 +16022,28 @@
     </row>
     <row r="331" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A331" t="s">
-        <v>1321</v>
+        <v>1322</v>
       </c>
       <c r="B331" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="C331" t="s">
-        <v>20</v>
+        <v>739</v>
       </c>
       <c r="D331" t="s">
         <v>161</v>
       </c>
       <c r="E331" s="1" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="F331" s="1" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
       <c r="G331" t="s">
         <v>10</v>
       </c>
       <c r="H331" t="s">
-        <v>909</v>
+        <v>10</v>
       </c>
       <c r="I331" t="s">
         <v>10</v>
@@ -16060,22 +16054,22 @@
     </row>
     <row r="332" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A332" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="B332" t="s">
+        <v>1328</v>
+      </c>
+      <c r="C332" t="s">
+        <v>88</v>
+      </c>
+      <c r="D332" t="s">
+        <v>1329</v>
+      </c>
+      <c r="E332" s="1" t="s">
         <v>1327</v>
       </c>
-      <c r="C332" t="s">
-        <v>739</v>
-      </c>
-      <c r="D332" t="s">
-        <v>161</v>
-      </c>
-      <c r="E332" s="1" t="s">
-        <v>1326</v>
-      </c>
       <c r="F332" s="1" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="G332" t="s">
         <v>10</v>
@@ -16092,28 +16086,28 @@
     </row>
     <row r="333" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A333" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="B333" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C333" t="s">
+        <v>36</v>
+      </c>
+      <c r="D333" t="s">
+        <v>791</v>
+      </c>
+      <c r="E333" s="1" t="s">
         <v>1331</v>
       </c>
-      <c r="C333" t="s">
-        <v>88</v>
-      </c>
-      <c r="D333" t="s">
+      <c r="F333" s="1" t="s">
         <v>1332</v>
       </c>
-      <c r="E333" s="1" t="s">
-        <v>1330</v>
-      </c>
-      <c r="F333" s="1" t="s">
-        <v>1330</v>
-      </c>
-      <c r="G333" t="s">
-        <v>10</v>
+      <c r="G333" s="1" t="s">
+        <v>1333</v>
       </c>
       <c r="H333" t="s">
-        <v>10</v>
+        <v>1334</v>
       </c>
       <c r="I333" t="s">
         <v>10</v>
@@ -16124,28 +16118,28 @@
     </row>
     <row r="334" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A334" t="s">
-        <v>1333</v>
+        <v>1335</v>
       </c>
       <c r="B334" t="s">
-        <v>1316</v>
+        <v>1337</v>
       </c>
       <c r="C334" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D334" t="s">
-        <v>791</v>
+        <v>70</v>
       </c>
       <c r="E334" s="1" t="s">
-        <v>1334</v>
+        <v>1336</v>
       </c>
       <c r="F334" s="1" t="s">
-        <v>1335</v>
-      </c>
-      <c r="G334" s="1" t="s">
-        <v>1336</v>
+        <v>1338</v>
+      </c>
+      <c r="G334" t="s">
+        <v>10</v>
       </c>
       <c r="H334" t="s">
-        <v>1337</v>
+        <v>10</v>
       </c>
       <c r="I334" t="s">
         <v>10</v>
@@ -16156,28 +16150,28 @@
     </row>
     <row r="335" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A335" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B335" t="s">
-        <v>1340</v>
+        <v>69</v>
       </c>
       <c r="C335" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="D335" t="s">
         <v>70</v>
       </c>
       <c r="E335" s="1" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="F335" s="1" t="s">
+        <v>1340</v>
+      </c>
+      <c r="G335" t="s">
+        <v>10</v>
+      </c>
+      <c r="H335" t="s">
         <v>1341</v>
-      </c>
-      <c r="G335" t="s">
-        <v>10</v>
-      </c>
-      <c r="H335" t="s">
-        <v>10</v>
       </c>
       <c r="I335" t="s">
         <v>10</v>
@@ -16191,13 +16185,13 @@
         <v>1342</v>
       </c>
       <c r="B336" t="s">
-        <v>69</v>
+        <v>1344</v>
       </c>
       <c r="C336" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D336" t="s">
-        <v>70</v>
+        <v>221</v>
       </c>
       <c r="E336" s="1" t="s">
         <v>1343</v>
@@ -16209,7 +16203,7 @@
         <v>10</v>
       </c>
       <c r="H336" t="s">
-        <v>1344</v>
+        <v>10</v>
       </c>
       <c r="I336" t="s">
         <v>10</v>
@@ -16226,22 +16220,22 @@
         <v>1347</v>
       </c>
       <c r="C337" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="D337" t="s">
-        <v>221</v>
+        <v>70</v>
       </c>
       <c r="E337" s="1" t="s">
         <v>1346</v>
       </c>
       <c r="F337" s="1" t="s">
-        <v>1346</v>
+        <v>1348</v>
       </c>
       <c r="G337" t="s">
         <v>10</v>
       </c>
       <c r="H337" t="s">
-        <v>10</v>
+        <v>1349</v>
       </c>
       <c r="I337" t="s">
         <v>10</v>
@@ -16252,31 +16246,31 @@
     </row>
     <row r="338" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A338" t="s">
-        <v>1348</v>
+        <v>1350</v>
       </c>
       <c r="B338" t="s">
-        <v>1350</v>
+        <v>1617</v>
       </c>
       <c r="C338" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D338" t="s">
         <v>70</v>
       </c>
       <c r="E338" s="1" t="s">
-        <v>1349</v>
-      </c>
-      <c r="F338" s="1" t="s">
         <v>1351</v>
       </c>
+      <c r="F338" t="s">
+        <v>10</v>
+      </c>
       <c r="G338" t="s">
         <v>10</v>
       </c>
       <c r="H338" t="s">
-        <v>1352</v>
+        <v>10</v>
       </c>
       <c r="I338" t="s">
-        <v>10</v>
+        <v>1350</v>
       </c>
       <c r="J338" t="s">
         <v>10</v>
@@ -16284,10 +16278,10 @@
     </row>
     <row r="339" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A339" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="B339" t="s">
-        <v>1620</v>
+        <v>1354</v>
       </c>
       <c r="C339" t="s">
         <v>20</v>
@@ -16296,10 +16290,10 @@
         <v>70</v>
       </c>
       <c r="E339" s="1" t="s">
-        <v>1354</v>
-      </c>
-      <c r="F339" t="s">
-        <v>10</v>
+        <v>1353</v>
+      </c>
+      <c r="F339" s="1" t="s">
+        <v>1355</v>
       </c>
       <c r="G339" t="s">
         <v>10</v>
@@ -16308,7 +16302,7 @@
         <v>10</v>
       </c>
       <c r="I339" t="s">
-        <v>1353</v>
+        <v>10</v>
       </c>
       <c r="J339" t="s">
         <v>10</v>
@@ -16316,28 +16310,28 @@
     </row>
     <row r="340" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A340" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="B340" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="C340" t="s">
-        <v>20</v>
+        <v>739</v>
       </c>
       <c r="D340" t="s">
         <v>70</v>
       </c>
       <c r="E340" s="1" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="F340" s="1" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="G340" t="s">
         <v>10</v>
       </c>
       <c r="H340" t="s">
-        <v>10</v>
+        <v>1359</v>
       </c>
       <c r="I340" t="s">
         <v>10</v>
@@ -16348,28 +16342,28 @@
     </row>
     <row r="341" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A341" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="B341" t="s">
+        <v>1362</v>
+      </c>
+      <c r="C341" t="s">
+        <v>1364</v>
+      </c>
+      <c r="D341" t="s">
+        <v>112</v>
+      </c>
+      <c r="E341" s="1" t="s">
         <v>1361</v>
       </c>
-      <c r="C341" t="s">
-        <v>739</v>
-      </c>
-      <c r="D341" t="s">
-        <v>70</v>
-      </c>
-      <c r="E341" s="1" t="s">
-        <v>1360</v>
-      </c>
       <c r="F341" s="1" t="s">
-        <v>1360</v>
+        <v>1363</v>
       </c>
       <c r="G341" t="s">
         <v>10</v>
       </c>
       <c r="H341" t="s">
-        <v>1362</v>
+        <v>10</v>
       </c>
       <c r="I341" t="s">
         <v>10</v>
@@ -16380,31 +16374,31 @@
     </row>
     <row r="342" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A342" t="s">
-        <v>1363</v>
+        <v>1365</v>
       </c>
       <c r="B342" t="s">
-        <v>1365</v>
+        <v>1671</v>
       </c>
       <c r="C342" t="s">
+        <v>20</v>
+      </c>
+      <c r="D342" t="s">
+        <v>161</v>
+      </c>
+      <c r="E342" s="1" t="s">
+        <v>1366</v>
+      </c>
+      <c r="F342" t="s">
+        <v>10</v>
+      </c>
+      <c r="G342" t="s">
+        <v>10</v>
+      </c>
+      <c r="H342" t="s">
+        <v>10</v>
+      </c>
+      <c r="I342" t="s">
         <v>1367</v>
-      </c>
-      <c r="D342" t="s">
-        <v>112</v>
-      </c>
-      <c r="E342" s="1" t="s">
-        <v>1364</v>
-      </c>
-      <c r="F342" s="1" t="s">
-        <v>1366</v>
-      </c>
-      <c r="G342" t="s">
-        <v>10</v>
-      </c>
-      <c r="H342" t="s">
-        <v>10</v>
-      </c>
-      <c r="I342" t="s">
-        <v>10</v>
       </c>
       <c r="J342" t="s">
         <v>10</v>
@@ -16415,28 +16409,28 @@
         <v>1368</v>
       </c>
       <c r="B343" t="s">
-        <v>1674</v>
+        <v>1370</v>
       </c>
       <c r="C343" t="s">
         <v>20</v>
       </c>
       <c r="D343" t="s">
-        <v>161</v>
+        <v>70</v>
       </c>
       <c r="E343" s="1" t="s">
         <v>1369</v>
       </c>
-      <c r="F343" t="s">
-        <v>10</v>
+      <c r="F343" s="1" t="s">
+        <v>1371</v>
       </c>
       <c r="G343" t="s">
         <v>10</v>
       </c>
       <c r="H343" t="s">
-        <v>10</v>
+        <v>1372</v>
       </c>
       <c r="I343" t="s">
-        <v>1370</v>
+        <v>10</v>
       </c>
       <c r="J343" t="s">
         <v>10</v>
@@ -16444,10 +16438,10 @@
     </row>
     <row r="344" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A344" t="s">
-        <v>1371</v>
+        <v>1373</v>
       </c>
       <c r="B344" t="s">
-        <v>1373</v>
+        <v>1375</v>
       </c>
       <c r="C344" t="s">
         <v>20</v>
@@ -16456,16 +16450,16 @@
         <v>70</v>
       </c>
       <c r="E344" s="1" t="s">
-        <v>1372</v>
+        <v>1374</v>
       </c>
       <c r="F344" s="1" t="s">
-        <v>1374</v>
+        <v>1376</v>
       </c>
       <c r="G344" t="s">
         <v>10</v>
       </c>
       <c r="H344" t="s">
-        <v>1375</v>
+        <v>1377</v>
       </c>
       <c r="I344" t="s">
         <v>10</v>
@@ -16476,19 +16470,19 @@
     </row>
     <row r="345" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A345" t="s">
-        <v>1376</v>
+        <v>1378</v>
       </c>
       <c r="B345" t="s">
-        <v>1378</v>
+        <v>1694</v>
       </c>
       <c r="C345" t="s">
         <v>20</v>
       </c>
       <c r="D345" t="s">
-        <v>70</v>
+        <v>407</v>
       </c>
       <c r="E345" s="1" t="s">
-        <v>1377</v>
+        <v>1379</v>
       </c>
       <c r="F345" s="1" t="s">
         <v>1379</v>
@@ -16497,7 +16491,7 @@
         <v>10</v>
       </c>
       <c r="H345" t="s">
-        <v>1380</v>
+        <v>10</v>
       </c>
       <c r="I345" t="s">
         <v>10</v>
@@ -16508,22 +16502,22 @@
     </row>
     <row r="346" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A346" t="s">
+        <v>1380</v>
+      </c>
+      <c r="B346" t="s">
+        <v>1382</v>
+      </c>
+      <c r="C346" t="s">
+        <v>20</v>
+      </c>
+      <c r="D346" t="s">
+        <v>1622</v>
+      </c>
+      <c r="E346" s="1" t="s">
         <v>1381</v>
       </c>
-      <c r="B346" t="s">
-        <v>1697</v>
-      </c>
-      <c r="C346" t="s">
-        <v>20</v>
-      </c>
-      <c r="D346" t="s">
-        <v>407</v>
-      </c>
-      <c r="E346" s="1" t="s">
-        <v>1382</v>
-      </c>
-      <c r="F346" s="1" t="s">
-        <v>1382</v>
+      <c r="F346" t="s">
+        <v>10</v>
       </c>
       <c r="G346" t="s">
         <v>10</v>
@@ -16543,25 +16537,25 @@
         <v>1383</v>
       </c>
       <c r="B347" t="s">
+        <v>209</v>
+      </c>
+      <c r="C347" t="s">
+        <v>36</v>
+      </c>
+      <c r="D347" t="s">
+        <v>70</v>
+      </c>
+      <c r="E347" t="s">
+        <v>10</v>
+      </c>
+      <c r="F347" s="1" t="s">
+        <v>1384</v>
+      </c>
+      <c r="G347" t="s">
+        <v>10</v>
+      </c>
+      <c r="H347" t="s">
         <v>1385</v>
-      </c>
-      <c r="C347" t="s">
-        <v>20</v>
-      </c>
-      <c r="D347" t="s">
-        <v>1625</v>
-      </c>
-      <c r="E347" s="1" t="s">
-        <v>1384</v>
-      </c>
-      <c r="F347" t="s">
-        <v>10</v>
-      </c>
-      <c r="G347" t="s">
-        <v>10</v>
-      </c>
-      <c r="H347" t="s">
-        <v>10</v>
       </c>
       <c r="I347" t="s">
         <v>10</v>
@@ -16575,25 +16569,25 @@
         <v>1386</v>
       </c>
       <c r="B348" t="s">
-        <v>209</v>
+        <v>1388</v>
       </c>
       <c r="C348" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D348" t="s">
-        <v>70</v>
-      </c>
-      <c r="E348" t="s">
-        <v>10</v>
+        <v>83</v>
+      </c>
+      <c r="E348" s="1" t="s">
+        <v>1387</v>
       </c>
       <c r="F348" s="1" t="s">
-        <v>1387</v>
+        <v>1389</v>
       </c>
       <c r="G348" t="s">
         <v>10</v>
       </c>
       <c r="H348" t="s">
-        <v>1388</v>
+        <v>1390</v>
       </c>
       <c r="I348" t="s">
         <v>10</v>
@@ -16604,28 +16598,28 @@
     </row>
     <row r="349" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A349" t="s">
-        <v>1389</v>
+        <v>1391</v>
       </c>
       <c r="B349" t="s">
-        <v>1391</v>
+        <v>1393</v>
       </c>
       <c r="C349" t="s">
         <v>20</v>
       </c>
       <c r="D349" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="E349" s="1" t="s">
-        <v>1390</v>
+        <v>1392</v>
       </c>
       <c r="F349" s="1" t="s">
-        <v>1392</v>
+        <v>1394</v>
       </c>
       <c r="G349" t="s">
         <v>10</v>
       </c>
       <c r="H349" t="s">
-        <v>1393</v>
+        <v>1395</v>
       </c>
       <c r="I349" t="s">
         <v>10</v>
@@ -16636,31 +16630,31 @@
     </row>
     <row r="350" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A350" t="s">
-        <v>1394</v>
+        <v>1396</v>
       </c>
       <c r="B350" t="s">
-        <v>1396</v>
+        <v>1398</v>
       </c>
       <c r="C350" t="s">
         <v>20</v>
       </c>
       <c r="D350" t="s">
-        <v>70</v>
+        <v>407</v>
       </c>
       <c r="E350" s="1" t="s">
-        <v>1395</v>
-      </c>
-      <c r="F350" s="1" t="s">
         <v>1397</v>
       </c>
+      <c r="F350" t="s">
+        <v>10</v>
+      </c>
       <c r="G350" t="s">
         <v>10</v>
       </c>
       <c r="H350" t="s">
-        <v>1398</v>
+        <v>10</v>
       </c>
       <c r="I350" t="s">
-        <v>10</v>
+        <v>1399</v>
       </c>
       <c r="J350" t="s">
         <v>10</v>
@@ -16668,22 +16662,22 @@
     </row>
     <row r="351" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A351" t="s">
-        <v>1399</v>
+        <v>1401</v>
       </c>
       <c r="B351" t="s">
-        <v>1401</v>
+        <v>69</v>
       </c>
       <c r="C351" t="s">
         <v>20</v>
       </c>
       <c r="D351" t="s">
-        <v>407</v>
+        <v>70</v>
       </c>
       <c r="E351" s="1" t="s">
         <v>1400</v>
       </c>
-      <c r="F351" t="s">
-        <v>10</v>
+      <c r="F351" s="1" t="s">
+        <v>1402</v>
       </c>
       <c r="G351" t="s">
         <v>10</v>
@@ -16692,7 +16686,7 @@
         <v>10</v>
       </c>
       <c r="I351" t="s">
-        <v>1402</v>
+        <v>10</v>
       </c>
       <c r="J351" t="s">
         <v>10</v>
@@ -16700,22 +16694,22 @@
     </row>
     <row r="352" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A352" t="s">
+        <v>1403</v>
+      </c>
+      <c r="B352" t="s">
+        <v>1405</v>
+      </c>
+      <c r="C352" t="s">
+        <v>20</v>
+      </c>
+      <c r="D352" t="s">
+        <v>407</v>
+      </c>
+      <c r="E352" s="1" t="s">
         <v>1404</v>
       </c>
-      <c r="B352" t="s">
-        <v>69</v>
-      </c>
-      <c r="C352" t="s">
-        <v>20</v>
-      </c>
-      <c r="D352" t="s">
-        <v>70</v>
-      </c>
-      <c r="E352" s="1" t="s">
-        <v>1403</v>
-      </c>
-      <c r="F352" s="1" t="s">
-        <v>1405</v>
+      <c r="F352" t="s">
+        <v>10</v>
       </c>
       <c r="G352" t="s">
         <v>10</v>
@@ -16724,7 +16718,7 @@
         <v>10</v>
       </c>
       <c r="I352" t="s">
-        <v>10</v>
+        <v>374</v>
       </c>
       <c r="J352" t="s">
         <v>10</v>
@@ -16741,13 +16735,13 @@
         <v>20</v>
       </c>
       <c r="D353" t="s">
-        <v>407</v>
+        <v>75</v>
       </c>
       <c r="E353" s="1" t="s">
         <v>1407</v>
       </c>
-      <c r="F353" t="s">
-        <v>10</v>
+      <c r="F353" s="1" t="s">
+        <v>1409</v>
       </c>
       <c r="G353" t="s">
         <v>10</v>
@@ -16756,7 +16750,7 @@
         <v>10</v>
       </c>
       <c r="I353" t="s">
-        <v>374</v>
+        <v>10</v>
       </c>
       <c r="J353" t="s">
         <v>10</v>
@@ -16764,22 +16758,22 @@
     </row>
     <row r="354" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
-        <v>1409</v>
+        <v>1410</v>
       </c>
       <c r="B354" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C354" t="s">
+        <v>20</v>
+      </c>
+      <c r="D354" t="s">
+        <v>83</v>
+      </c>
+      <c r="E354" s="1" t="s">
         <v>1411</v>
       </c>
-      <c r="C354" t="s">
-        <v>20</v>
-      </c>
-      <c r="D354" t="s">
-        <v>75</v>
-      </c>
-      <c r="E354" s="1" t="s">
-        <v>1410</v>
-      </c>
-      <c r="F354" s="1" t="s">
-        <v>1412</v>
+      <c r="F354" t="s">
+        <v>10</v>
       </c>
       <c r="G354" t="s">
         <v>10</v>
@@ -16788,7 +16782,7 @@
         <v>10</v>
       </c>
       <c r="I354" t="s">
-        <v>10</v>
+        <v>1413</v>
       </c>
       <c r="J354" t="s">
         <v>10</v>
@@ -16796,20 +16790,20 @@
     </row>
     <row r="355" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A355" t="s">
-        <v>1413</v>
+        <v>1414</v>
       </c>
       <c r="B355" t="s">
+        <v>1416</v>
+      </c>
+      <c r="C355" t="s">
+        <v>20</v>
+      </c>
+      <c r="D355" t="s">
+        <v>1672</v>
+      </c>
+      <c r="E355" s="1" t="s">
         <v>1415</v>
       </c>
-      <c r="C355" t="s">
-        <v>20</v>
-      </c>
-      <c r="D355" t="s">
-        <v>83</v>
-      </c>
-      <c r="E355" s="1" t="s">
-        <v>1414</v>
-      </c>
       <c r="F355" t="s">
         <v>10</v>
       </c>
@@ -16820,7 +16814,7 @@
         <v>10</v>
       </c>
       <c r="I355" t="s">
-        <v>1416</v>
+        <v>1417</v>
       </c>
       <c r="J355" t="s">
         <v>10</v>
@@ -16828,31 +16822,31 @@
     </row>
     <row r="356" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A356" t="s">
-        <v>1417</v>
+        <v>1418</v>
       </c>
       <c r="B356" t="s">
+        <v>1420</v>
+      </c>
+      <c r="C356" t="s">
+        <v>20</v>
+      </c>
+      <c r="D356" t="s">
+        <v>75</v>
+      </c>
+      <c r="E356" s="1" t="s">
         <v>1419</v>
       </c>
-      <c r="C356" t="s">
-        <v>20</v>
-      </c>
-      <c r="D356" t="s">
-        <v>1675</v>
-      </c>
-      <c r="E356" s="1" t="s">
-        <v>1418</v>
-      </c>
-      <c r="F356" t="s">
-        <v>10</v>
+      <c r="F356" s="1" t="s">
+        <v>1421</v>
       </c>
       <c r="G356" t="s">
         <v>10</v>
       </c>
       <c r="H356" t="s">
-        <v>10</v>
+        <v>1422</v>
       </c>
       <c r="I356" t="s">
-        <v>1420</v>
+        <v>10</v>
       </c>
       <c r="J356" t="s">
         <v>10</v>
@@ -16860,28 +16854,28 @@
     </row>
     <row r="357" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A357" t="s">
-        <v>1421</v>
+        <v>1423</v>
       </c>
       <c r="B357" t="s">
-        <v>1423</v>
+        <v>1425</v>
       </c>
       <c r="C357" t="s">
         <v>20</v>
       </c>
       <c r="D357" t="s">
-        <v>75</v>
+        <v>1019</v>
       </c>
       <c r="E357" s="1" t="s">
-        <v>1422</v>
+        <v>1424</v>
       </c>
       <c r="F357" s="1" t="s">
-        <v>1424</v>
+        <v>1426</v>
       </c>
       <c r="G357" t="s">
         <v>10</v>
       </c>
       <c r="H357" t="s">
-        <v>1425</v>
+        <v>1427</v>
       </c>
       <c r="I357" t="s">
         <v>10</v>
@@ -16892,28 +16886,28 @@
     </row>
     <row r="358" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A358" t="s">
-        <v>1426</v>
+        <v>1428</v>
       </c>
       <c r="B358" t="s">
-        <v>1428</v>
+        <v>1430</v>
       </c>
       <c r="C358" t="s">
         <v>20</v>
       </c>
       <c r="D358" t="s">
-        <v>1019</v>
+        <v>31</v>
       </c>
       <c r="E358" s="1" t="s">
-        <v>1427</v>
+        <v>1429</v>
       </c>
       <c r="F358" s="1" t="s">
-        <v>1429</v>
+        <v>1431</v>
       </c>
       <c r="G358" t="s">
         <v>10</v>
       </c>
       <c r="H358" t="s">
-        <v>1430</v>
+        <v>10</v>
       </c>
       <c r="I358" t="s">
         <v>10</v>
@@ -16924,7 +16918,7 @@
     </row>
     <row r="359" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A359" t="s">
-        <v>1431</v>
+        <v>1432</v>
       </c>
       <c r="B359" t="s">
         <v>1433</v>
@@ -16933,10 +16927,10 @@
         <v>20</v>
       </c>
       <c r="D359" t="s">
-        <v>31</v>
+        <v>1435</v>
       </c>
       <c r="E359" s="1" t="s">
-        <v>1432</v>
+        <v>1429</v>
       </c>
       <c r="F359" s="1" t="s">
         <v>1434</v>
@@ -16945,7 +16939,7 @@
         <v>10</v>
       </c>
       <c r="H359" t="s">
-        <v>10</v>
+        <v>1436</v>
       </c>
       <c r="I359" t="s">
         <v>10</v>
@@ -16956,31 +16950,31 @@
     </row>
     <row r="360" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A360" t="s">
-        <v>1435</v>
+        <v>1437</v>
       </c>
       <c r="B360" t="s">
-        <v>1436</v>
+        <v>1439</v>
       </c>
       <c r="C360" t="s">
         <v>20</v>
       </c>
       <c r="D360" t="s">
+        <v>287</v>
+      </c>
+      <c r="E360" s="1" t="s">
         <v>1438</v>
       </c>
-      <c r="E360" s="1" t="s">
-        <v>1432</v>
-      </c>
-      <c r="F360" s="1" t="s">
-        <v>1437</v>
+      <c r="F360" t="s">
+        <v>10</v>
       </c>
       <c r="G360" t="s">
         <v>10</v>
       </c>
       <c r="H360" t="s">
-        <v>1439</v>
+        <v>10</v>
       </c>
       <c r="I360" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="J360" t="s">
         <v>10</v>
@@ -16997,7 +16991,7 @@
         <v>20</v>
       </c>
       <c r="D361" t="s">
-        <v>287</v>
+        <v>31</v>
       </c>
       <c r="E361" s="1" t="s">
         <v>1441</v>
@@ -17012,7 +17006,7 @@
         <v>10</v>
       </c>
       <c r="I361" t="s">
-        <v>66</v>
+        <v>1443</v>
       </c>
       <c r="J361" t="s">
         <v>10</v>
@@ -17020,31 +17014,31 @@
     </row>
     <row r="362" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A362" t="s">
-        <v>1443</v>
+        <v>1444</v>
       </c>
       <c r="B362" t="s">
+        <v>1446</v>
+      </c>
+      <c r="C362" t="s">
+        <v>20</v>
+      </c>
+      <c r="D362" t="s">
+        <v>343</v>
+      </c>
+      <c r="E362" s="1" t="s">
         <v>1445</v>
       </c>
-      <c r="C362" t="s">
-        <v>20</v>
-      </c>
-      <c r="D362" t="s">
-        <v>31</v>
-      </c>
-      <c r="E362" s="1" t="s">
-        <v>1444</v>
-      </c>
-      <c r="F362" t="s">
-        <v>10</v>
+      <c r="F362" s="1" t="s">
+        <v>1445</v>
       </c>
       <c r="G362" t="s">
         <v>10</v>
       </c>
       <c r="H362" t="s">
-        <v>10</v>
+        <v>1447</v>
       </c>
       <c r="I362" t="s">
-        <v>1446</v>
+        <v>10</v>
       </c>
       <c r="J362" t="s">
         <v>10</v>
@@ -17052,10 +17046,10 @@
     </row>
     <row r="363" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A363" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
       <c r="B363" t="s">
-        <v>1449</v>
+        <v>1450</v>
       </c>
       <c r="C363" t="s">
         <v>20</v>
@@ -17064,16 +17058,16 @@
         <v>343</v>
       </c>
       <c r="E363" s="1" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
       <c r="F363" s="1" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
       <c r="G363" t="s">
         <v>10</v>
       </c>
       <c r="H363" t="s">
-        <v>1450</v>
+        <v>1447</v>
       </c>
       <c r="I363" t="s">
         <v>10</v>
@@ -17105,7 +17099,7 @@
         <v>10</v>
       </c>
       <c r="H364" t="s">
-        <v>1450</v>
+        <v>1447</v>
       </c>
       <c r="I364" t="s">
         <v>10</v>
@@ -17137,7 +17131,7 @@
         <v>10</v>
       </c>
       <c r="H365" t="s">
-        <v>1450</v>
+        <v>1447</v>
       </c>
       <c r="I365" t="s">
         <v>10</v>
@@ -17169,7 +17163,7 @@
         <v>10</v>
       </c>
       <c r="H366" t="s">
-        <v>1450</v>
+        <v>1447</v>
       </c>
       <c r="I366" t="s">
         <v>10</v>
@@ -17201,7 +17195,7 @@
         <v>10</v>
       </c>
       <c r="H367" t="s">
-        <v>1450</v>
+        <v>1447</v>
       </c>
       <c r="I367" t="s">
         <v>10</v>
@@ -17215,31 +17209,31 @@
         <v>1463</v>
       </c>
       <c r="B368" t="s">
-        <v>1465</v>
+        <v>1618</v>
       </c>
       <c r="C368" t="s">
         <v>20</v>
       </c>
       <c r="D368" t="s">
-        <v>343</v>
+        <v>31</v>
       </c>
       <c r="E368" s="1" t="s">
         <v>1464</v>
       </c>
-      <c r="F368" s="1" t="s">
-        <v>1464</v>
+      <c r="F368" t="s">
+        <v>10</v>
       </c>
       <c r="G368" t="s">
         <v>10</v>
       </c>
       <c r="H368" t="s">
-        <v>1450</v>
+        <v>10</v>
       </c>
       <c r="I368" t="s">
-        <v>10</v>
+        <v>1465</v>
       </c>
       <c r="J368" t="s">
-        <v>10</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="369" spans="1:10" x14ac:dyDescent="0.2">
@@ -17247,54 +17241,54 @@
         <v>1466</v>
       </c>
       <c r="B369" t="s">
-        <v>1621</v>
+        <v>1468</v>
       </c>
       <c r="C369" t="s">
         <v>20</v>
       </c>
       <c r="D369" t="s">
-        <v>31</v>
+        <v>308</v>
       </c>
       <c r="E369" s="1" t="s">
+        <v>1619</v>
+      </c>
+      <c r="F369" s="1" t="s">
         <v>1467</v>
       </c>
-      <c r="F369" t="s">
-        <v>10</v>
-      </c>
-      <c r="G369" t="s">
-        <v>10</v>
+      <c r="G369" s="1" t="s">
+        <v>1469</v>
       </c>
       <c r="H369" t="s">
         <v>10</v>
       </c>
       <c r="I369" t="s">
-        <v>1468</v>
+        <v>10</v>
       </c>
       <c r="J369" t="s">
-        <v>1468</v>
+        <v>10</v>
       </c>
     </row>
     <row r="370" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A370" t="s">
-        <v>1469</v>
+        <v>1470</v>
       </c>
       <c r="B370" t="s">
+        <v>1472</v>
+      </c>
+      <c r="C370" t="s">
+        <v>36</v>
+      </c>
+      <c r="D370" t="s">
+        <v>112</v>
+      </c>
+      <c r="E370" s="1" t="s">
         <v>1471</v>
       </c>
-      <c r="C370" t="s">
-        <v>20</v>
-      </c>
-      <c r="D370" t="s">
-        <v>308</v>
-      </c>
-      <c r="E370" s="1" t="s">
-        <v>1622</v>
-      </c>
       <c r="F370" s="1" t="s">
-        <v>1470</v>
-      </c>
-      <c r="G370" s="1" t="s">
-        <v>1472</v>
+        <v>1471</v>
+      </c>
+      <c r="G370" t="s">
+        <v>10</v>
       </c>
       <c r="H370" t="s">
         <v>10</v>
@@ -17314,16 +17308,16 @@
         <v>1475</v>
       </c>
       <c r="C371" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D371" t="s">
-        <v>112</v>
+        <v>1685</v>
       </c>
       <c r="E371" s="1" t="s">
         <v>1474</v>
       </c>
-      <c r="F371" s="1" t="s">
-        <v>1474</v>
+      <c r="F371" t="s">
+        <v>10</v>
       </c>
       <c r="G371" t="s">
         <v>10</v>
@@ -17343,13 +17337,13 @@
         <v>1476</v>
       </c>
       <c r="B372" t="s">
-        <v>1478</v>
+        <v>1673</v>
       </c>
       <c r="C372" t="s">
         <v>20</v>
       </c>
       <c r="D372" t="s">
-        <v>1688</v>
+        <v>1674</v>
       </c>
       <c r="E372" s="1" t="s">
         <v>1477</v>
@@ -17364,7 +17358,7 @@
         <v>10</v>
       </c>
       <c r="I372" t="s">
-        <v>10</v>
+        <v>1478</v>
       </c>
       <c r="J372" t="s">
         <v>10</v>
@@ -17375,28 +17369,28 @@
         <v>1479</v>
       </c>
       <c r="B373" t="s">
-        <v>1676</v>
+        <v>1481</v>
       </c>
       <c r="C373" t="s">
         <v>20</v>
       </c>
       <c r="D373" t="s">
-        <v>1677</v>
+        <v>198</v>
       </c>
       <c r="E373" s="1" t="s">
         <v>1480</v>
       </c>
-      <c r="F373" t="s">
-        <v>10</v>
-      </c>
-      <c r="G373" t="s">
-        <v>10</v>
+      <c r="F373" s="1" t="s">
+        <v>1480</v>
+      </c>
+      <c r="G373" s="1" t="s">
+        <v>1482</v>
       </c>
       <c r="H373" t="s">
-        <v>10</v>
+        <v>1483</v>
       </c>
       <c r="I373" t="s">
-        <v>1481</v>
+        <v>1483</v>
       </c>
       <c r="J373" t="s">
         <v>10</v>
@@ -17404,31 +17398,31 @@
     </row>
     <row r="374" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A374" t="s">
-        <v>1482</v>
+        <v>1484</v>
       </c>
       <c r="B374" t="s">
-        <v>1484</v>
+        <v>1486</v>
       </c>
       <c r="C374" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="D374" t="s">
-        <v>198</v>
+        <v>75</v>
       </c>
       <c r="E374" s="1" t="s">
-        <v>1483</v>
-      </c>
-      <c r="F374" s="1" t="s">
-        <v>1483</v>
-      </c>
-      <c r="G374" s="1" t="s">
         <v>1485</v>
       </c>
+      <c r="F374" t="s">
+        <v>10</v>
+      </c>
+      <c r="G374" t="s">
+        <v>10</v>
+      </c>
       <c r="H374" t="s">
-        <v>1486</v>
+        <v>10</v>
       </c>
       <c r="I374" t="s">
-        <v>1486</v>
+        <v>10</v>
       </c>
       <c r="J374" t="s">
         <v>10</v>
@@ -17445,7 +17439,7 @@
         <v>36</v>
       </c>
       <c r="D375" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E375" s="1" t="s">
         <v>1488</v>
@@ -17477,19 +17471,19 @@
         <v>36</v>
       </c>
       <c r="D376" t="s">
-        <v>70</v>
+        <v>1495</v>
       </c>
       <c r="E376" s="1" t="s">
         <v>1491</v>
       </c>
-      <c r="F376" t="s">
-        <v>10</v>
-      </c>
-      <c r="G376" t="s">
-        <v>10</v>
+      <c r="F376" s="1" t="s">
+        <v>1493</v>
+      </c>
+      <c r="G376" s="1" t="s">
+        <v>1494</v>
       </c>
       <c r="H376" t="s">
-        <v>10</v>
+        <v>1496</v>
       </c>
       <c r="I376" t="s">
         <v>10</v>
@@ -17500,28 +17494,28 @@
     </row>
     <row r="377" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A377" t="s">
-        <v>1493</v>
+        <v>1498</v>
       </c>
       <c r="B377" t="s">
-        <v>1495</v>
+        <v>1499</v>
       </c>
       <c r="C377" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D377" t="s">
-        <v>1498</v>
+        <v>1685</v>
       </c>
       <c r="E377" s="1" t="s">
-        <v>1494</v>
+        <v>1497</v>
       </c>
       <c r="F377" s="1" t="s">
-        <v>1496</v>
-      </c>
-      <c r="G377" s="1" t="s">
-        <v>1497</v>
+        <v>1500</v>
+      </c>
+      <c r="G377" t="s">
+        <v>10</v>
       </c>
       <c r="H377" t="s">
-        <v>1499</v>
+        <v>10</v>
       </c>
       <c r="I377" t="s">
         <v>10</v>
@@ -17535,25 +17529,25 @@
         <v>1501</v>
       </c>
       <c r="B378" t="s">
+        <v>1503</v>
+      </c>
+      <c r="C378" t="s">
+        <v>36</v>
+      </c>
+      <c r="D378" t="s">
+        <v>70</v>
+      </c>
+      <c r="E378" s="1" t="s">
         <v>1502</v>
       </c>
-      <c r="C378" t="s">
-        <v>20</v>
-      </c>
-      <c r="D378" t="s">
-        <v>1688</v>
-      </c>
-      <c r="E378" s="1" t="s">
-        <v>1500</v>
-      </c>
       <c r="F378" s="1" t="s">
-        <v>1503</v>
+        <v>1502</v>
       </c>
       <c r="G378" t="s">
         <v>10</v>
       </c>
       <c r="H378" t="s">
-        <v>10</v>
+        <v>1504</v>
       </c>
       <c r="I378" t="s">
         <v>10</v>
@@ -17564,28 +17558,28 @@
     </row>
     <row r="379" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A379" t="s">
-        <v>1504</v>
+        <v>1505</v>
       </c>
       <c r="B379" t="s">
+        <v>1507</v>
+      </c>
+      <c r="C379" t="s">
+        <v>20</v>
+      </c>
+      <c r="D379" t="s">
+        <v>75</v>
+      </c>
+      <c r="E379" s="1" t="s">
         <v>1506</v>
       </c>
-      <c r="C379" t="s">
-        <v>36</v>
-      </c>
-      <c r="D379" t="s">
-        <v>70</v>
-      </c>
-      <c r="E379" s="1" t="s">
-        <v>1505</v>
-      </c>
       <c r="F379" s="1" t="s">
-        <v>1505</v>
+        <v>1508</v>
       </c>
       <c r="G379" t="s">
         <v>10</v>
       </c>
       <c r="H379" t="s">
-        <v>1507</v>
+        <v>66</v>
       </c>
       <c r="I379" t="s">
         <v>10</v>
@@ -17596,28 +17590,28 @@
     </row>
     <row r="380" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A380" t="s">
-        <v>1508</v>
+        <v>1509</v>
       </c>
       <c r="B380" t="s">
-        <v>1510</v>
+        <v>1511</v>
       </c>
       <c r="C380" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="D380" t="s">
         <v>75</v>
       </c>
       <c r="E380" s="1" t="s">
-        <v>1509</v>
+        <v>1510</v>
       </c>
       <c r="F380" s="1" t="s">
-        <v>1511</v>
+        <v>1512</v>
       </c>
       <c r="G380" t="s">
         <v>10</v>
       </c>
       <c r="H380" t="s">
-        <v>66</v>
+        <v>1513</v>
       </c>
       <c r="I380" t="s">
         <v>10</v>
@@ -17628,28 +17622,28 @@
     </row>
     <row r="381" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A381" t="s">
-        <v>1512</v>
+        <v>1514</v>
       </c>
       <c r="B381" t="s">
-        <v>1514</v>
+        <v>1516</v>
       </c>
       <c r="C381" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="D381" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E381" s="1" t="s">
-        <v>1513</v>
+        <v>1515</v>
       </c>
       <c r="F381" s="1" t="s">
         <v>1515</v>
       </c>
-      <c r="G381" t="s">
-        <v>10</v>
+      <c r="G381" s="1" t="s">
+        <v>1517</v>
       </c>
       <c r="H381" t="s">
-        <v>1516</v>
+        <v>10</v>
       </c>
       <c r="I381" t="s">
         <v>10</v>
@@ -17660,31 +17654,31 @@
     </row>
     <row r="382" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A382" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
       <c r="B382" t="s">
+        <v>1620</v>
+      </c>
+      <c r="C382" t="s">
+        <v>20</v>
+      </c>
+      <c r="D382" t="s">
+        <v>1622</v>
+      </c>
+      <c r="E382" s="1" t="s">
         <v>1519</v>
       </c>
-      <c r="C382" t="s">
-        <v>47</v>
-      </c>
-      <c r="D382" t="s">
-        <v>83</v>
-      </c>
-      <c r="E382" s="1" t="s">
-        <v>1518</v>
-      </c>
-      <c r="F382" s="1" t="s">
-        <v>1518</v>
-      </c>
-      <c r="G382" s="1" t="s">
+      <c r="F382" t="s">
+        <v>10</v>
+      </c>
+      <c r="G382" t="s">
+        <v>10</v>
+      </c>
+      <c r="H382" t="s">
+        <v>10</v>
+      </c>
+      <c r="I382" t="s">
         <v>1520</v>
-      </c>
-      <c r="H382" t="s">
-        <v>10</v>
-      </c>
-      <c r="I382" t="s">
-        <v>10</v>
       </c>
       <c r="J382" t="s">
         <v>10</v>
@@ -17695,13 +17689,13 @@
         <v>1521</v>
       </c>
       <c r="B383" t="s">
-        <v>1623</v>
+        <v>1523</v>
       </c>
       <c r="C383" t="s">
         <v>20</v>
       </c>
       <c r="D383" t="s">
-        <v>1625</v>
+        <v>161</v>
       </c>
       <c r="E383" s="1" t="s">
         <v>1522</v>
@@ -17716,7 +17710,7 @@
         <v>10</v>
       </c>
       <c r="I383" t="s">
-        <v>1523</v>
+        <v>1524</v>
       </c>
       <c r="J383" t="s">
         <v>10</v>
@@ -17724,20 +17718,20 @@
     </row>
     <row r="384" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A384" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="B384" t="s">
+        <v>1527</v>
+      </c>
+      <c r="C384" t="s">
+        <v>20</v>
+      </c>
+      <c r="D384" t="s">
+        <v>83</v>
+      </c>
+      <c r="E384" s="1" t="s">
         <v>1526</v>
       </c>
-      <c r="C384" t="s">
-        <v>20</v>
-      </c>
-      <c r="D384" t="s">
-        <v>161</v>
-      </c>
-      <c r="E384" s="1" t="s">
-        <v>1525</v>
-      </c>
       <c r="F384" t="s">
         <v>10</v>
       </c>
@@ -17748,7 +17742,7 @@
         <v>10</v>
       </c>
       <c r="I384" t="s">
-        <v>1527</v>
+        <v>1528</v>
       </c>
       <c r="J384" t="s">
         <v>10</v>
@@ -17756,31 +17750,31 @@
     </row>
     <row r="385" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A385" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="B385" t="s">
+        <v>69</v>
+      </c>
+      <c r="C385" t="s">
+        <v>36</v>
+      </c>
+      <c r="D385" t="s">
+        <v>70</v>
+      </c>
+      <c r="E385" s="1" t="s">
         <v>1530</v>
       </c>
-      <c r="C385" t="s">
-        <v>20</v>
-      </c>
-      <c r="D385" t="s">
-        <v>83</v>
-      </c>
-      <c r="E385" s="1" t="s">
-        <v>1529</v>
-      </c>
-      <c r="F385" t="s">
-        <v>10</v>
+      <c r="F385" s="1" t="s">
+        <v>1530</v>
       </c>
       <c r="G385" t="s">
         <v>10</v>
       </c>
       <c r="H385" t="s">
-        <v>10</v>
+        <v>1531</v>
       </c>
       <c r="I385" t="s">
-        <v>1531</v>
+        <v>10</v>
       </c>
       <c r="J385" t="s">
         <v>10</v>
@@ -17791,25 +17785,25 @@
         <v>1532</v>
       </c>
       <c r="B386" t="s">
-        <v>69</v>
+        <v>1534</v>
       </c>
       <c r="C386" t="s">
         <v>36</v>
       </c>
       <c r="D386" t="s">
-        <v>70</v>
+        <v>407</v>
       </c>
       <c r="E386" s="1" t="s">
         <v>1533</v>
       </c>
       <c r="F386" s="1" t="s">
-        <v>1533</v>
+        <v>1535</v>
       </c>
       <c r="G386" t="s">
         <v>10</v>
       </c>
       <c r="H386" t="s">
-        <v>1534</v>
+        <v>10</v>
       </c>
       <c r="I386" t="s">
         <v>10</v>
@@ -17820,22 +17814,22 @@
     </row>
     <row r="387" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A387" t="s">
-        <v>1535</v>
+        <v>1536</v>
       </c>
       <c r="B387" t="s">
+        <v>671</v>
+      </c>
+      <c r="C387" t="s">
+        <v>20</v>
+      </c>
+      <c r="D387" t="s">
+        <v>31</v>
+      </c>
+      <c r="E387" s="1" t="s">
+        <v>670</v>
+      </c>
+      <c r="F387" s="1" t="s">
         <v>1537</v>
-      </c>
-      <c r="C387" t="s">
-        <v>36</v>
-      </c>
-      <c r="D387" t="s">
-        <v>407</v>
-      </c>
-      <c r="E387" s="1" t="s">
-        <v>1536</v>
-      </c>
-      <c r="F387" s="1" t="s">
-        <v>1538</v>
       </c>
       <c r="G387" t="s">
         <v>10</v>
@@ -17852,22 +17846,22 @@
     </row>
     <row r="388" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A388" t="s">
+        <v>1538</v>
+      </c>
+      <c r="B388" t="s">
+        <v>1540</v>
+      </c>
+      <c r="C388" t="s">
+        <v>20</v>
+      </c>
+      <c r="D388" t="s">
+        <v>1033</v>
+      </c>
+      <c r="E388" s="1" t="s">
         <v>1539</v>
       </c>
-      <c r="B388" t="s">
-        <v>671</v>
-      </c>
-      <c r="C388" t="s">
-        <v>20</v>
-      </c>
-      <c r="D388" t="s">
-        <v>31</v>
-      </c>
-      <c r="E388" s="1" t="s">
-        <v>670</v>
-      </c>
       <c r="F388" s="1" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="G388" t="s">
         <v>10</v>
@@ -17893,16 +17887,16 @@
         <v>20</v>
       </c>
       <c r="D389" t="s">
-        <v>1033</v>
+        <v>1495</v>
       </c>
       <c r="E389" s="1" t="s">
         <v>1542</v>
       </c>
       <c r="F389" s="1" t="s">
-        <v>1542</v>
-      </c>
-      <c r="G389" t="s">
-        <v>10</v>
+        <v>1544</v>
+      </c>
+      <c r="G389" s="1" t="s">
+        <v>1545</v>
       </c>
       <c r="H389" t="s">
         <v>10</v>
@@ -17916,25 +17910,25 @@
     </row>
     <row r="390" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A390" t="s">
-        <v>1544</v>
+        <v>1546</v>
       </c>
       <c r="B390" t="s">
-        <v>1546</v>
+        <v>1548</v>
       </c>
       <c r="C390" t="s">
         <v>20</v>
       </c>
       <c r="D390" t="s">
-        <v>1498</v>
+        <v>83</v>
       </c>
       <c r="E390" s="1" t="s">
-        <v>1545</v>
+        <v>1547</v>
       </c>
       <c r="F390" s="1" t="s">
-        <v>1547</v>
+        <v>1549</v>
       </c>
       <c r="G390" s="1" t="s">
-        <v>1548</v>
+        <v>1550</v>
       </c>
       <c r="H390" t="s">
         <v>10</v>
@@ -17948,28 +17942,28 @@
     </row>
     <row r="391" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A391" t="s">
-        <v>1549</v>
+        <v>1551</v>
       </c>
       <c r="B391" t="s">
-        <v>1551</v>
+        <v>1553</v>
       </c>
       <c r="C391" t="s">
         <v>20</v>
       </c>
       <c r="D391" t="s">
-        <v>83</v>
+        <v>198</v>
       </c>
       <c r="E391" s="1" t="s">
-        <v>1550</v>
+        <v>1552</v>
       </c>
       <c r="F391" s="1" t="s">
-        <v>1552</v>
-      </c>
-      <c r="G391" s="1" t="s">
-        <v>1553</v>
+        <v>1554</v>
+      </c>
+      <c r="G391" t="s">
+        <v>10</v>
       </c>
       <c r="H391" t="s">
-        <v>10</v>
+        <v>1555</v>
       </c>
       <c r="I391" t="s">
         <v>10</v>
@@ -17980,10 +17974,10 @@
     </row>
     <row r="392" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A392" t="s">
-        <v>1554</v>
+        <v>1556</v>
       </c>
       <c r="B392" t="s">
-        <v>1556</v>
+        <v>1558</v>
       </c>
       <c r="C392" t="s">
         <v>20</v>
@@ -17992,19 +17986,19 @@
         <v>198</v>
       </c>
       <c r="E392" s="1" t="s">
-        <v>1555</v>
-      </c>
-      <c r="F392" s="1" t="s">
         <v>1557</v>
       </c>
+      <c r="F392" t="s">
+        <v>10</v>
+      </c>
       <c r="G392" t="s">
         <v>10</v>
       </c>
       <c r="H392" t="s">
-        <v>1558</v>
+        <v>10</v>
       </c>
       <c r="I392" t="s">
-        <v>10</v>
+        <v>1559</v>
       </c>
       <c r="J392" t="s">
         <v>10</v>
@@ -18012,10 +18006,10 @@
     </row>
     <row r="393" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A393" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="B393" t="s">
-        <v>1561</v>
+        <v>1675</v>
       </c>
       <c r="C393" t="s">
         <v>20</v>
@@ -18024,7 +18018,7 @@
         <v>198</v>
       </c>
       <c r="E393" s="1" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
       <c r="F393" t="s">
         <v>10</v>
@@ -18047,28 +18041,28 @@
         <v>1563</v>
       </c>
       <c r="B394" t="s">
-        <v>1678</v>
+        <v>1565</v>
       </c>
       <c r="C394" t="s">
         <v>20</v>
       </c>
       <c r="D394" t="s">
-        <v>198</v>
+        <v>83</v>
       </c>
       <c r="E394" s="1" t="s">
         <v>1564</v>
       </c>
-      <c r="F394" t="s">
-        <v>10</v>
+      <c r="F394" s="1" t="s">
+        <v>1564</v>
       </c>
       <c r="G394" t="s">
         <v>10</v>
       </c>
       <c r="H394" t="s">
-        <v>10</v>
+        <v>1427</v>
       </c>
       <c r="I394" t="s">
-        <v>1565</v>
+        <v>1427</v>
       </c>
       <c r="J394" t="s">
         <v>10</v>
@@ -18079,28 +18073,28 @@
         <v>1566</v>
       </c>
       <c r="B395" t="s">
-        <v>1568</v>
+        <v>1676</v>
       </c>
       <c r="C395" t="s">
         <v>20</v>
       </c>
       <c r="D395" t="s">
-        <v>83</v>
+        <v>407</v>
       </c>
       <c r="E395" s="1" t="s">
         <v>1567</v>
       </c>
-      <c r="F395" s="1" t="s">
-        <v>1567</v>
+      <c r="F395" t="s">
+        <v>10</v>
       </c>
       <c r="G395" t="s">
         <v>10</v>
       </c>
       <c r="H395" t="s">
-        <v>1430</v>
+        <v>10</v>
       </c>
       <c r="I395" t="s">
-        <v>1430</v>
+        <v>1568</v>
       </c>
       <c r="J395" t="s">
         <v>10</v>
@@ -18111,28 +18105,28 @@
         <v>1569</v>
       </c>
       <c r="B396" t="s">
-        <v>1679</v>
+        <v>1571</v>
       </c>
       <c r="C396" t="s">
-        <v>20</v>
+        <v>1573</v>
       </c>
       <c r="D396" t="s">
-        <v>407</v>
+        <v>657</v>
       </c>
       <c r="E396" s="1" t="s">
         <v>1570</v>
       </c>
-      <c r="F396" t="s">
-        <v>10</v>
-      </c>
-      <c r="G396" t="s">
-        <v>10</v>
+      <c r="F396" s="1" t="s">
+        <v>1570</v>
+      </c>
+      <c r="G396" s="1" t="s">
+        <v>1572</v>
       </c>
       <c r="H396" t="s">
         <v>10</v>
       </c>
       <c r="I396" t="s">
-        <v>1571</v>
+        <v>10</v>
       </c>
       <c r="J396" t="s">
         <v>10</v>
@@ -18140,25 +18134,25 @@
     </row>
     <row r="397" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A397" t="s">
-        <v>1572</v>
+        <v>1574</v>
       </c>
       <c r="B397" t="s">
-        <v>1574</v>
+        <v>1576</v>
       </c>
       <c r="C397" t="s">
-        <v>1576</v>
+        <v>20</v>
       </c>
       <c r="D397" t="s">
-        <v>657</v>
+        <v>407</v>
       </c>
       <c r="E397" s="1" t="s">
-        <v>1573</v>
+        <v>1575</v>
       </c>
       <c r="F397" s="1" t="s">
-        <v>1573</v>
-      </c>
-      <c r="G397" s="1" t="s">
         <v>1575</v>
+      </c>
+      <c r="G397" t="s">
+        <v>10</v>
       </c>
       <c r="H397" t="s">
         <v>10</v>
@@ -18181,13 +18175,13 @@
         <v>20</v>
       </c>
       <c r="D398" t="s">
-        <v>407</v>
+        <v>1677</v>
       </c>
       <c r="E398" s="1" t="s">
         <v>1578</v>
       </c>
-      <c r="F398" s="1" t="s">
-        <v>1578</v>
+      <c r="F398" t="s">
+        <v>10</v>
       </c>
       <c r="G398" t="s">
         <v>10</v>
@@ -18196,7 +18190,7 @@
         <v>10</v>
       </c>
       <c r="I398" t="s">
-        <v>10</v>
+        <v>1146</v>
       </c>
       <c r="J398" t="s">
         <v>10</v>
@@ -18213,7 +18207,7 @@
         <v>20</v>
       </c>
       <c r="D399" t="s">
-        <v>1680</v>
+        <v>407</v>
       </c>
       <c r="E399" s="1" t="s">
         <v>1581</v>
@@ -18228,7 +18222,7 @@
         <v>10</v>
       </c>
       <c r="I399" t="s">
-        <v>1146</v>
+        <v>10</v>
       </c>
       <c r="J399" t="s">
         <v>10</v>
@@ -18245,7 +18239,7 @@
         <v>20</v>
       </c>
       <c r="D400" t="s">
-        <v>407</v>
+        <v>1677</v>
       </c>
       <c r="E400" s="1" t="s">
         <v>1584</v>
@@ -18260,7 +18254,7 @@
         <v>10</v>
       </c>
       <c r="I400" t="s">
-        <v>10</v>
+        <v>1586</v>
       </c>
       <c r="J400" t="s">
         <v>10</v>
@@ -18268,20 +18262,20 @@
     </row>
     <row r="401" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A401" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="B401" t="s">
+        <v>1589</v>
+      </c>
+      <c r="C401" t="s">
+        <v>20</v>
+      </c>
+      <c r="D401" t="s">
+        <v>407</v>
+      </c>
+      <c r="E401" s="1" t="s">
         <v>1588</v>
       </c>
-      <c r="C401" t="s">
-        <v>20</v>
-      </c>
-      <c r="D401" t="s">
-        <v>1680</v>
-      </c>
-      <c r="E401" s="1" t="s">
-        <v>1587</v>
-      </c>
       <c r="F401" t="s">
         <v>10</v>
       </c>
@@ -18292,7 +18286,7 @@
         <v>10</v>
       </c>
       <c r="I401" t="s">
-        <v>1589</v>
+        <v>10</v>
       </c>
       <c r="J401" t="s">
         <v>10</v>
@@ -18306,16 +18300,16 @@
         <v>1592</v>
       </c>
       <c r="C402" t="s">
-        <v>20</v>
+        <v>1593</v>
       </c>
       <c r="D402" t="s">
-        <v>407</v>
+        <v>270</v>
       </c>
       <c r="E402" s="1" t="s">
         <v>1591</v>
       </c>
-      <c r="F402" t="s">
-        <v>10</v>
+      <c r="F402" s="1" t="s">
+        <v>1591</v>
       </c>
       <c r="G402" t="s">
         <v>10</v>
@@ -18332,22 +18326,22 @@
     </row>
     <row r="403" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A403" t="s">
-        <v>1593</v>
+        <v>1594</v>
       </c>
       <c r="B403" t="s">
-        <v>1595</v>
+        <v>1596</v>
       </c>
       <c r="C403" t="s">
-        <v>1596</v>
+        <v>20</v>
       </c>
       <c r="D403" t="s">
         <v>270</v>
       </c>
       <c r="E403" s="1" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
       <c r="F403" s="1" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
       <c r="G403" t="s">
         <v>10</v>
@@ -18373,13 +18367,13 @@
         <v>20</v>
       </c>
       <c r="D404" t="s">
-        <v>270</v>
+        <v>407</v>
       </c>
       <c r="E404" s="1" t="s">
         <v>1598</v>
       </c>
-      <c r="F404" s="1" t="s">
-        <v>1598</v>
+      <c r="F404" t="s">
+        <v>10</v>
       </c>
       <c r="G404" t="s">
         <v>10</v>
@@ -18402,16 +18396,16 @@
         <v>1602</v>
       </c>
       <c r="C405" t="s">
-        <v>20</v>
+        <v>900</v>
       </c>
       <c r="D405" t="s">
-        <v>407</v>
+        <v>758</v>
       </c>
       <c r="E405" s="1" t="s">
         <v>1601</v>
       </c>
-      <c r="F405" t="s">
-        <v>10</v>
+      <c r="F405" s="1" t="s">
+        <v>1601</v>
       </c>
       <c r="G405" t="s">
         <v>10</v>
@@ -18428,59 +18422,27 @@
     </row>
     <row r="406" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A406" t="s">
-        <v>1603</v>
+        <v>1679</v>
       </c>
       <c r="B406" t="s">
-        <v>1605</v>
+        <v>1680</v>
       </c>
       <c r="C406" t="s">
-        <v>900</v>
+        <v>1681</v>
       </c>
       <c r="D406" t="s">
-        <v>758</v>
+        <v>31</v>
       </c>
       <c r="E406" s="1" t="s">
-        <v>1604</v>
-      </c>
-      <c r="F406" s="1" t="s">
-        <v>1604</v>
-      </c>
-      <c r="G406" t="s">
-        <v>10</v>
-      </c>
-      <c r="H406" t="s">
-        <v>10</v>
-      </c>
-      <c r="I406" t="s">
-        <v>10</v>
-      </c>
-      <c r="J406" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="407" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A407" t="s">
+        <v>1683</v>
+      </c>
+      <c r="F406" t="s">
         <v>1682</v>
       </c>
-      <c r="B407" t="s">
-        <v>1683</v>
-      </c>
-      <c r="C407" t="s">
-        <v>1684</v>
-      </c>
-      <c r="D407" t="s">
-        <v>31</v>
-      </c>
-      <c r="E407" s="1" t="s">
-        <v>1686</v>
-      </c>
-      <c r="F407" t="s">
-        <v>1685</v>
-      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J406">
-    <sortCondition ref="A2:A406"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J405">
+    <sortCondition ref="A2:A405"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -18889,346 +18851,343 @@
     <hyperlink ref="E214" r:id="rId404" xr:uid="{00000000-0004-0000-0000-000091020000}"/>
     <hyperlink ref="F214" r:id="rId405" xr:uid="{00000000-0004-0000-0000-000092020000}"/>
     <hyperlink ref="E215" r:id="rId406" display="https://github.com/pavijovi3/OMNIC-FTIR-data-processing-tool" xr:uid="{00000000-0004-0000-0000-0000BC020000}"/>
-    <hyperlink ref="E216" r:id="rId407" xr:uid="{00000000-0004-0000-0000-0000C6020000}"/>
-    <hyperlink ref="F216" r:id="rId408" xr:uid="{00000000-0004-0000-0000-0000C7020000}"/>
-    <hyperlink ref="E217" r:id="rId409" xr:uid="{00000000-0004-0000-0000-0000C8020000}"/>
-    <hyperlink ref="F217" r:id="rId410" xr:uid="{00000000-0004-0000-0000-0000C9020000}"/>
-    <hyperlink ref="G217" r:id="rId411" xr:uid="{00000000-0004-0000-0000-0000CA020000}"/>
-    <hyperlink ref="E218" r:id="rId412" xr:uid="{00000000-0004-0000-0000-0000CB020000}"/>
-    <hyperlink ref="E219" r:id="rId413" xr:uid="{00000000-0004-0000-0000-0000CC020000}"/>
-    <hyperlink ref="F219" r:id="rId414" xr:uid="{00000000-0004-0000-0000-0000CD020000}"/>
-    <hyperlink ref="E220" r:id="rId415" xr:uid="{00000000-0004-0000-0000-0000CE020000}"/>
-    <hyperlink ref="F220" r:id="rId416" xr:uid="{00000000-0004-0000-0000-0000CF020000}"/>
-    <hyperlink ref="E221" r:id="rId417" xr:uid="{00000000-0004-0000-0000-0000D1020000}"/>
-    <hyperlink ref="F221" r:id="rId418" xr:uid="{00000000-0004-0000-0000-0000D2020000}"/>
-    <hyperlink ref="E222" r:id="rId419" xr:uid="{00000000-0004-0000-0000-0000D3020000}"/>
-    <hyperlink ref="E223" r:id="rId420" xr:uid="{00000000-0004-0000-0000-0000D5020000}"/>
-    <hyperlink ref="F223" r:id="rId421" xr:uid="{00000000-0004-0000-0000-0000D6020000}"/>
-    <hyperlink ref="E224" r:id="rId422" xr:uid="{00000000-0004-0000-0000-0000D9020000}"/>
-    <hyperlink ref="F224" r:id="rId423" xr:uid="{00000000-0004-0000-0000-0000DA020000}"/>
-    <hyperlink ref="G224" r:id="rId424" xr:uid="{00000000-0004-0000-0000-0000DB020000}"/>
-    <hyperlink ref="E225" r:id="rId425" xr:uid="{00000000-0004-0000-0000-0000DC020000}"/>
-    <hyperlink ref="F225" r:id="rId426" xr:uid="{00000000-0004-0000-0000-0000DD020000}"/>
-    <hyperlink ref="G225" r:id="rId427" xr:uid="{00000000-0004-0000-0000-0000DE020000}"/>
-    <hyperlink ref="E226" r:id="rId428" xr:uid="{00000000-0004-0000-0000-0000E0020000}"/>
-    <hyperlink ref="F226" r:id="rId429" xr:uid="{00000000-0004-0000-0000-0000E1020000}"/>
-    <hyperlink ref="E227" r:id="rId430" xr:uid="{00000000-0004-0000-0000-0000E3020000}"/>
-    <hyperlink ref="F227" r:id="rId431" xr:uid="{00000000-0004-0000-0000-0000E4020000}"/>
-    <hyperlink ref="E228" r:id="rId432" xr:uid="{00000000-0004-0000-0000-0000E6020000}"/>
-    <hyperlink ref="E229" r:id="rId433" xr:uid="{00000000-0004-0000-0000-0000E7020000}"/>
-    <hyperlink ref="E230" r:id="rId434" xr:uid="{00000000-0004-0000-0000-0000E8020000}"/>
-    <hyperlink ref="E231" r:id="rId435" xr:uid="{00000000-0004-0000-0000-0000E9020000}"/>
-    <hyperlink ref="F231" r:id="rId436" xr:uid="{00000000-0004-0000-0000-0000EA020000}"/>
-    <hyperlink ref="E232" r:id="rId437" xr:uid="{00000000-0004-0000-0000-0000EB020000}"/>
-    <hyperlink ref="F232" r:id="rId438" xr:uid="{00000000-0004-0000-0000-0000EC020000}"/>
-    <hyperlink ref="E233" r:id="rId439" xr:uid="{00000000-0004-0000-0000-0000EF020000}"/>
-    <hyperlink ref="F233" r:id="rId440" xr:uid="{00000000-0004-0000-0000-0000F0020000}"/>
-    <hyperlink ref="E234" r:id="rId441" xr:uid="{00000000-0004-0000-0000-0000F1020000}"/>
-    <hyperlink ref="F234" r:id="rId442" xr:uid="{00000000-0004-0000-0000-0000F2020000}"/>
-    <hyperlink ref="G234" r:id="rId443" xr:uid="{00000000-0004-0000-0000-0000F3020000}"/>
-    <hyperlink ref="E235" r:id="rId444" xr:uid="{00000000-0004-0000-0000-0000F4020000}"/>
-    <hyperlink ref="F235" r:id="rId445" xr:uid="{00000000-0004-0000-0000-0000F5020000}"/>
-    <hyperlink ref="E236" r:id="rId446" xr:uid="{00000000-0004-0000-0000-0000F8020000}"/>
-    <hyperlink ref="F236" r:id="rId447" xr:uid="{00000000-0004-0000-0000-0000F9020000}"/>
-    <hyperlink ref="G236" r:id="rId448" xr:uid="{00000000-0004-0000-0000-0000FA020000}"/>
-    <hyperlink ref="E237" r:id="rId449" xr:uid="{00000000-0004-0000-0000-0000FE020000}"/>
-    <hyperlink ref="F237" r:id="rId450" xr:uid="{00000000-0004-0000-0000-0000FF020000}"/>
-    <hyperlink ref="G237" r:id="rId451" xr:uid="{00000000-0004-0000-0000-000000030000}"/>
-    <hyperlink ref="E238" r:id="rId452" xr:uid="{00000000-0004-0000-0000-000001030000}"/>
-    <hyperlink ref="F238" r:id="rId453" xr:uid="{00000000-0004-0000-0000-000002030000}"/>
-    <hyperlink ref="G238" r:id="rId454" xr:uid="{00000000-0004-0000-0000-000003030000}"/>
-    <hyperlink ref="E239" r:id="rId455" display="https://github.com/NRCan/PlotFTIR" xr:uid="{00000000-0004-0000-0000-000006030000}"/>
-    <hyperlink ref="E240" r:id="rId456" xr:uid="{00000000-0004-0000-0000-00000B030000}"/>
-    <hyperlink ref="F240" r:id="rId457" xr:uid="{00000000-0004-0000-0000-00000C030000}"/>
-    <hyperlink ref="E241" r:id="rId458" xr:uid="{00000000-0004-0000-0000-00000D030000}"/>
-    <hyperlink ref="E242" r:id="rId459" xr:uid="{00000000-0004-0000-0000-00000F030000}"/>
-    <hyperlink ref="F242" r:id="rId460" xr:uid="{00000000-0004-0000-0000-000010030000}"/>
-    <hyperlink ref="G242" r:id="rId461" xr:uid="{00000000-0004-0000-0000-000011030000}"/>
-    <hyperlink ref="E243" r:id="rId462" xr:uid="{00000000-0004-0000-0000-000012030000}"/>
-    <hyperlink ref="F243" r:id="rId463" xr:uid="{00000000-0004-0000-0000-000013030000}"/>
-    <hyperlink ref="G243" r:id="rId464" xr:uid="{00000000-0004-0000-0000-000014030000}"/>
-    <hyperlink ref="E244" r:id="rId465" xr:uid="{00000000-0004-0000-0000-00001E030000}"/>
-    <hyperlink ref="E245" r:id="rId466" xr:uid="{00000000-0004-0000-0000-00001F030000}"/>
-    <hyperlink ref="F245" r:id="rId467" xr:uid="{00000000-0004-0000-0000-000020030000}"/>
-    <hyperlink ref="E246" r:id="rId468" xr:uid="{00000000-0004-0000-0000-000022030000}"/>
-    <hyperlink ref="E247" r:id="rId469" xr:uid="{00000000-0004-0000-0000-000025030000}"/>
-    <hyperlink ref="E248" r:id="rId470" xr:uid="{00000000-0004-0000-0000-000026030000}"/>
-    <hyperlink ref="E249" r:id="rId471" xr:uid="{00000000-0004-0000-0000-000027030000}"/>
-    <hyperlink ref="F249" r:id="rId472" xr:uid="{00000000-0004-0000-0000-000028030000}"/>
-    <hyperlink ref="E250" r:id="rId473" xr:uid="{00000000-0004-0000-0000-00002C030000}"/>
-    <hyperlink ref="F250" r:id="rId474" xr:uid="{00000000-0004-0000-0000-00002D030000}"/>
-    <hyperlink ref="E251" r:id="rId475" xr:uid="{00000000-0004-0000-0000-000030030000}"/>
-    <hyperlink ref="F251" r:id="rId476" xr:uid="{00000000-0004-0000-0000-000031030000}"/>
-    <hyperlink ref="E252" r:id="rId477" xr:uid="{00000000-0004-0000-0000-000034030000}"/>
-    <hyperlink ref="F252" r:id="rId478" xr:uid="{00000000-0004-0000-0000-000035030000}"/>
-    <hyperlink ref="E253" r:id="rId479" xr:uid="{00000000-0004-0000-0000-000036030000}"/>
-    <hyperlink ref="F253" r:id="rId480" xr:uid="{00000000-0004-0000-0000-000037030000}"/>
-    <hyperlink ref="G253" r:id="rId481" xr:uid="{00000000-0004-0000-0000-000038030000}"/>
-    <hyperlink ref="E254" r:id="rId482" xr:uid="{00000000-0004-0000-0000-00003B030000}"/>
-    <hyperlink ref="E255" r:id="rId483" xr:uid="{00000000-0004-0000-0000-00003C030000}"/>
-    <hyperlink ref="E256" r:id="rId484" xr:uid="{00000000-0004-0000-0000-00003D030000}"/>
-    <hyperlink ref="E257" r:id="rId485" xr:uid="{00000000-0004-0000-0000-000042030000}"/>
-    <hyperlink ref="F257" r:id="rId486" xr:uid="{00000000-0004-0000-0000-000043030000}"/>
-    <hyperlink ref="E258" r:id="rId487" xr:uid="{00000000-0004-0000-0000-000044030000}"/>
-    <hyperlink ref="F258" r:id="rId488" xr:uid="{00000000-0004-0000-0000-000045030000}"/>
-    <hyperlink ref="E259" r:id="rId489" xr:uid="{00000000-0004-0000-0000-00004B030000}"/>
-    <hyperlink ref="E260" r:id="rId490" xr:uid="{00000000-0004-0000-0000-00004C030000}"/>
-    <hyperlink ref="E261" r:id="rId491" xr:uid="{00000000-0004-0000-0000-00004D030000}"/>
-    <hyperlink ref="E262" r:id="rId492" xr:uid="{00000000-0004-0000-0000-000053030000}"/>
-    <hyperlink ref="F262" r:id="rId493" xr:uid="{00000000-0004-0000-0000-000054030000}"/>
-    <hyperlink ref="E263" r:id="rId494" xr:uid="{00000000-0004-0000-0000-000055030000}"/>
-    <hyperlink ref="E264" r:id="rId495" xr:uid="{00000000-0004-0000-0000-000056030000}"/>
-    <hyperlink ref="E265" r:id="rId496" xr:uid="{00000000-0004-0000-0000-000059030000}"/>
-    <hyperlink ref="F265" r:id="rId497" xr:uid="{00000000-0004-0000-0000-00005A030000}"/>
-    <hyperlink ref="E266" r:id="rId498" xr:uid="{00000000-0004-0000-0000-00005B030000}"/>
-    <hyperlink ref="F266" r:id="rId499" xr:uid="{00000000-0004-0000-0000-00005C030000}"/>
-    <hyperlink ref="E267" r:id="rId500" xr:uid="{00000000-0004-0000-0000-00005E030000}"/>
-    <hyperlink ref="F267" r:id="rId501" xr:uid="{00000000-0004-0000-0000-00005F030000}"/>
-    <hyperlink ref="E268" r:id="rId502" xr:uid="{00000000-0004-0000-0000-000060030000}"/>
-    <hyperlink ref="F268" r:id="rId503" xr:uid="{00000000-0004-0000-0000-000061030000}"/>
-    <hyperlink ref="E269" r:id="rId504" xr:uid="{00000000-0004-0000-0000-000062030000}"/>
-    <hyperlink ref="F269" r:id="rId505" xr:uid="{00000000-0004-0000-0000-000063030000}"/>
-    <hyperlink ref="E270" r:id="rId506" xr:uid="{00000000-0004-0000-0000-000064030000}"/>
-    <hyperlink ref="F270" r:id="rId507" xr:uid="{00000000-0004-0000-0000-000065030000}"/>
-    <hyperlink ref="E271" r:id="rId508" xr:uid="{00000000-0004-0000-0000-000067030000}"/>
-    <hyperlink ref="E272" r:id="rId509" xr:uid="{00000000-0004-0000-0000-00006B030000}"/>
-    <hyperlink ref="F272" r:id="rId510" xr:uid="{00000000-0004-0000-0000-00006C030000}"/>
-    <hyperlink ref="E274" r:id="rId511" xr:uid="{00000000-0004-0000-0000-00006E030000}"/>
-    <hyperlink ref="F274" r:id="rId512" xr:uid="{00000000-0004-0000-0000-00006F030000}"/>
-    <hyperlink ref="E275" r:id="rId513" xr:uid="{00000000-0004-0000-0000-000072030000}"/>
-    <hyperlink ref="F275" r:id="rId514" xr:uid="{00000000-0004-0000-0000-000073030000}"/>
-    <hyperlink ref="G275" r:id="rId515" location="!divAbstract" xr:uid="{00000000-0004-0000-0000-000074030000}"/>
-    <hyperlink ref="E276" r:id="rId516" xr:uid="{00000000-0004-0000-0000-000077030000}"/>
-    <hyperlink ref="F276" r:id="rId517" xr:uid="{00000000-0004-0000-0000-000078030000}"/>
-    <hyperlink ref="E277" r:id="rId518" xr:uid="{00000000-0004-0000-0000-000084030000}"/>
-    <hyperlink ref="F277" r:id="rId519" xr:uid="{00000000-0004-0000-0000-000085030000}"/>
-    <hyperlink ref="E278" r:id="rId520" xr:uid="{00000000-0004-0000-0000-000086030000}"/>
-    <hyperlink ref="F278" r:id="rId521" xr:uid="{00000000-0004-0000-0000-000087030000}"/>
-    <hyperlink ref="E279" r:id="rId522" xr:uid="{00000000-0004-0000-0000-000089030000}"/>
-    <hyperlink ref="F279" r:id="rId523" xr:uid="{00000000-0004-0000-0000-00008A030000}"/>
-    <hyperlink ref="G279" r:id="rId524" xr:uid="{00000000-0004-0000-0000-00008B030000}"/>
-    <hyperlink ref="E280" r:id="rId525" xr:uid="{00000000-0004-0000-0000-00008C030000}"/>
-    <hyperlink ref="F280" r:id="rId526" xr:uid="{00000000-0004-0000-0000-00008D030000}"/>
-    <hyperlink ref="E281" r:id="rId527" xr:uid="{00000000-0004-0000-0000-000094030000}"/>
-    <hyperlink ref="F281" r:id="rId528" xr:uid="{00000000-0004-0000-0000-000095030000}"/>
-    <hyperlink ref="E282" r:id="rId529" xr:uid="{00000000-0004-0000-0000-000096030000}"/>
-    <hyperlink ref="E283" r:id="rId530" xr:uid="{00000000-0004-0000-0000-000097030000}"/>
-    <hyperlink ref="E284" r:id="rId531" xr:uid="{00000000-0004-0000-0000-000098030000}"/>
-    <hyperlink ref="E285" r:id="rId532" xr:uid="{00000000-0004-0000-0000-00009B030000}"/>
-    <hyperlink ref="F285" r:id="rId533" xr:uid="{00000000-0004-0000-0000-00009C030000}"/>
-    <hyperlink ref="E286" r:id="rId534" xr:uid="{00000000-0004-0000-0000-00009D030000}"/>
-    <hyperlink ref="E287" r:id="rId535" xr:uid="{00000000-0004-0000-0000-00009F030000}"/>
-    <hyperlink ref="F287" r:id="rId536" xr:uid="{00000000-0004-0000-0000-0000A0030000}"/>
-    <hyperlink ref="E288" r:id="rId537" xr:uid="{00000000-0004-0000-0000-0000A1030000}"/>
-    <hyperlink ref="F288" r:id="rId538" xr:uid="{00000000-0004-0000-0000-0000A2030000}"/>
-    <hyperlink ref="E289" r:id="rId539" xr:uid="{00000000-0004-0000-0000-0000A3030000}"/>
-    <hyperlink ref="F289" r:id="rId540" xr:uid="{00000000-0004-0000-0000-0000A4030000}"/>
-    <hyperlink ref="E290" r:id="rId541" xr:uid="{00000000-0004-0000-0000-0000A6030000}"/>
-    <hyperlink ref="F290" r:id="rId542" xr:uid="{00000000-0004-0000-0000-0000A7030000}"/>
-    <hyperlink ref="E291" r:id="rId543" xr:uid="{00000000-0004-0000-0000-0000A8030000}"/>
-    <hyperlink ref="F291" r:id="rId544" xr:uid="{00000000-0004-0000-0000-0000A9030000}"/>
-    <hyperlink ref="E292" r:id="rId545" xr:uid="{00000000-0004-0000-0000-0000AA030000}"/>
-    <hyperlink ref="E293" r:id="rId546" xr:uid="{00000000-0004-0000-0000-0000AB030000}"/>
-    <hyperlink ref="E294" r:id="rId547" xr:uid="{00000000-0004-0000-0000-0000AC030000}"/>
-    <hyperlink ref="E295" r:id="rId548" xr:uid="{00000000-0004-0000-0000-0000AD030000}"/>
-    <hyperlink ref="F295" r:id="rId549" xr:uid="{00000000-0004-0000-0000-0000AE030000}"/>
-    <hyperlink ref="E296" r:id="rId550" xr:uid="{00000000-0004-0000-0000-0000B1030000}"/>
-    <hyperlink ref="F296" r:id="rId551" xr:uid="{00000000-0004-0000-0000-0000B2030000}"/>
-    <hyperlink ref="E297" r:id="rId552" xr:uid="{00000000-0004-0000-0000-0000B3030000}"/>
-    <hyperlink ref="E298" r:id="rId553" xr:uid="{00000000-0004-0000-0000-0000B4030000}"/>
-    <hyperlink ref="E299" r:id="rId554" xr:uid="{00000000-0004-0000-0000-0000B5030000}"/>
-    <hyperlink ref="F299" r:id="rId555" xr:uid="{00000000-0004-0000-0000-0000B6030000}"/>
-    <hyperlink ref="E300" r:id="rId556" xr:uid="{00000000-0004-0000-0000-0000B7030000}"/>
-    <hyperlink ref="E301" r:id="rId557" xr:uid="{00000000-0004-0000-0000-0000B8030000}"/>
-    <hyperlink ref="F301" r:id="rId558" xr:uid="{00000000-0004-0000-0000-0000B9030000}"/>
-    <hyperlink ref="E302" r:id="rId559" xr:uid="{00000000-0004-0000-0000-0000BA030000}"/>
-    <hyperlink ref="F302" r:id="rId560" xr:uid="{00000000-0004-0000-0000-0000BB030000}"/>
-    <hyperlink ref="E303" r:id="rId561" xr:uid="{00000000-0004-0000-0000-0000BC030000}"/>
-    <hyperlink ref="F303" r:id="rId562" xr:uid="{00000000-0004-0000-0000-0000BD030000}"/>
-    <hyperlink ref="E304" r:id="rId563" xr:uid="{00000000-0004-0000-0000-0000BF030000}"/>
-    <hyperlink ref="F304" r:id="rId564" xr:uid="{00000000-0004-0000-0000-0000C0030000}"/>
-    <hyperlink ref="E305" r:id="rId565" xr:uid="{00000000-0004-0000-0000-0000C1030000}"/>
-    <hyperlink ref="F305" r:id="rId566" xr:uid="{00000000-0004-0000-0000-0000C2030000}"/>
-    <hyperlink ref="E306" r:id="rId567" xr:uid="{00000000-0004-0000-0000-0000C4030000}"/>
-    <hyperlink ref="F306" r:id="rId568" xr:uid="{00000000-0004-0000-0000-0000C5030000}"/>
-    <hyperlink ref="E307" r:id="rId569" xr:uid="{00000000-0004-0000-0000-0000C6030000}"/>
-    <hyperlink ref="F307" r:id="rId570" xr:uid="{00000000-0004-0000-0000-0000C7030000}"/>
-    <hyperlink ref="E308" r:id="rId571" xr:uid="{00000000-0004-0000-0000-0000C8030000}"/>
-    <hyperlink ref="F308" r:id="rId572" xr:uid="{00000000-0004-0000-0000-0000C9030000}"/>
-    <hyperlink ref="E309" r:id="rId573" xr:uid="{00000000-0004-0000-0000-0000CA030000}"/>
-    <hyperlink ref="E310" r:id="rId574" xr:uid="{00000000-0004-0000-0000-0000CC030000}"/>
-    <hyperlink ref="F310" r:id="rId575" xr:uid="{00000000-0004-0000-0000-0000CD030000}"/>
-    <hyperlink ref="E311" r:id="rId576" xr:uid="{00000000-0004-0000-0000-0000CF030000}"/>
-    <hyperlink ref="F311" r:id="rId577" xr:uid="{00000000-0004-0000-0000-0000D0030000}"/>
-    <hyperlink ref="G311" r:id="rId578" xr:uid="{00000000-0004-0000-0000-0000D1030000}"/>
-    <hyperlink ref="E312" r:id="rId579" xr:uid="{00000000-0004-0000-0000-0000D2030000}"/>
-    <hyperlink ref="F312" r:id="rId580" xr:uid="{00000000-0004-0000-0000-0000D3030000}"/>
-    <hyperlink ref="E313" r:id="rId581" xr:uid="{00000000-0004-0000-0000-0000D4030000}"/>
-    <hyperlink ref="E314" r:id="rId582" xr:uid="{00000000-0004-0000-0000-0000D5030000}"/>
-    <hyperlink ref="E315" r:id="rId583" xr:uid="{00000000-0004-0000-0000-0000D6030000}"/>
-    <hyperlink ref="F315" r:id="rId584" xr:uid="{00000000-0004-0000-0000-0000D7030000}"/>
-    <hyperlink ref="E316" r:id="rId585" xr:uid="{00000000-0004-0000-0000-0000D8030000}"/>
-    <hyperlink ref="F316" r:id="rId586" xr:uid="{00000000-0004-0000-0000-0000D9030000}"/>
-    <hyperlink ref="F317" r:id="rId587" xr:uid="{00000000-0004-0000-0000-0000DE030000}"/>
-    <hyperlink ref="G317" r:id="rId588" xr:uid="{00000000-0004-0000-0000-0000DF030000}"/>
-    <hyperlink ref="E318" r:id="rId589" xr:uid="{00000000-0004-0000-0000-0000E0030000}"/>
-    <hyperlink ref="F318" r:id="rId590" xr:uid="{00000000-0004-0000-0000-0000E1030000}"/>
-    <hyperlink ref="G318" r:id="rId591" xr:uid="{00000000-0004-0000-0000-0000E2030000}"/>
-    <hyperlink ref="E319" r:id="rId592" xr:uid="{00000000-0004-0000-0000-0000EB030000}"/>
-    <hyperlink ref="F320" r:id="rId593" xr:uid="{00000000-0004-0000-0000-0000EC030000}"/>
-    <hyperlink ref="E321" r:id="rId594" xr:uid="{00000000-0004-0000-0000-0000F9030000}"/>
-    <hyperlink ref="F321" r:id="rId595" xr:uid="{00000000-0004-0000-0000-0000FA030000}"/>
-    <hyperlink ref="E322" r:id="rId596" xr:uid="{00000000-0004-0000-0000-0000FC030000}"/>
-    <hyperlink ref="F322" r:id="rId597" xr:uid="{00000000-0004-0000-0000-0000FD030000}"/>
-    <hyperlink ref="G322" r:id="rId598" xr:uid="{00000000-0004-0000-0000-0000FE030000}"/>
-    <hyperlink ref="E323" r:id="rId599" xr:uid="{00000000-0004-0000-0000-000002040000}"/>
-    <hyperlink ref="E324" r:id="rId600" xr:uid="{00000000-0004-0000-0000-000003040000}"/>
-    <hyperlink ref="E325" r:id="rId601" xr:uid="{00000000-0004-0000-0000-000005040000}"/>
-    <hyperlink ref="F325" r:id="rId602" xr:uid="{00000000-0004-0000-0000-000006040000}"/>
-    <hyperlink ref="E326" r:id="rId603" xr:uid="{00000000-0004-0000-0000-000007040000}"/>
-    <hyperlink ref="F326" r:id="rId604" xr:uid="{00000000-0004-0000-0000-000008040000}"/>
-    <hyperlink ref="E327" r:id="rId605" xr:uid="{00000000-0004-0000-0000-000009040000}"/>
-    <hyperlink ref="F327" r:id="rId606" xr:uid="{00000000-0004-0000-0000-00000A040000}"/>
-    <hyperlink ref="E328" r:id="rId607" xr:uid="{00000000-0004-0000-0000-00000C040000}"/>
-    <hyperlink ref="E329" r:id="rId608" xr:uid="{00000000-0004-0000-0000-00000F040000}"/>
-    <hyperlink ref="F329" r:id="rId609" xr:uid="{00000000-0004-0000-0000-000010040000}"/>
-    <hyperlink ref="G329" r:id="rId610" xr:uid="{00000000-0004-0000-0000-000011040000}"/>
-    <hyperlink ref="E330" r:id="rId611" xr:uid="{00000000-0004-0000-0000-000016040000}"/>
-    <hyperlink ref="E331" r:id="rId612" xr:uid="{00000000-0004-0000-0000-000019040000}"/>
-    <hyperlink ref="F331" r:id="rId613" xr:uid="{00000000-0004-0000-0000-00001A040000}"/>
-    <hyperlink ref="E332" r:id="rId614" xr:uid="{00000000-0004-0000-0000-00001B040000}"/>
-    <hyperlink ref="F332" r:id="rId615" xr:uid="{00000000-0004-0000-0000-00001C040000}"/>
-    <hyperlink ref="E333" r:id="rId616" xr:uid="{00000000-0004-0000-0000-00001D040000}"/>
-    <hyperlink ref="F333" r:id="rId617" xr:uid="{00000000-0004-0000-0000-00001E040000}"/>
-    <hyperlink ref="E334" r:id="rId618" xr:uid="{00000000-0004-0000-0000-000020040000}"/>
-    <hyperlink ref="F334" r:id="rId619" xr:uid="{00000000-0004-0000-0000-000021040000}"/>
-    <hyperlink ref="G334" r:id="rId620" xr:uid="{00000000-0004-0000-0000-000022040000}"/>
-    <hyperlink ref="E335" r:id="rId621" xr:uid="{00000000-0004-0000-0000-000024040000}"/>
-    <hyperlink ref="F335" r:id="rId622" xr:uid="{00000000-0004-0000-0000-000025040000}"/>
-    <hyperlink ref="E336" r:id="rId623" xr:uid="{00000000-0004-0000-0000-000026040000}"/>
-    <hyperlink ref="F336" r:id="rId624" xr:uid="{00000000-0004-0000-0000-000027040000}"/>
-    <hyperlink ref="E337" r:id="rId625" xr:uid="{00000000-0004-0000-0000-000028040000}"/>
-    <hyperlink ref="F337" r:id="rId626" xr:uid="{00000000-0004-0000-0000-000029040000}"/>
-    <hyperlink ref="E338" r:id="rId627" xr:uid="{00000000-0004-0000-0000-00002A040000}"/>
-    <hyperlink ref="F338" r:id="rId628" xr:uid="{00000000-0004-0000-0000-00002B040000}"/>
-    <hyperlink ref="E339" r:id="rId629" xr:uid="{00000000-0004-0000-0000-00002C040000}"/>
-    <hyperlink ref="E340" r:id="rId630" xr:uid="{00000000-0004-0000-0000-00002D040000}"/>
-    <hyperlink ref="F340" r:id="rId631" xr:uid="{00000000-0004-0000-0000-00002E040000}"/>
-    <hyperlink ref="E341" r:id="rId632" xr:uid="{00000000-0004-0000-0000-00002F040000}"/>
-    <hyperlink ref="F341" r:id="rId633" xr:uid="{00000000-0004-0000-0000-000030040000}"/>
-    <hyperlink ref="E342" r:id="rId634" xr:uid="{00000000-0004-0000-0000-000031040000}"/>
-    <hyperlink ref="F342" r:id="rId635" xr:uid="{00000000-0004-0000-0000-000032040000}"/>
-    <hyperlink ref="E343" r:id="rId636" xr:uid="{00000000-0004-0000-0000-000036040000}"/>
-    <hyperlink ref="E344" r:id="rId637" xr:uid="{00000000-0004-0000-0000-000037040000}"/>
-    <hyperlink ref="F344" r:id="rId638" xr:uid="{00000000-0004-0000-0000-000038040000}"/>
-    <hyperlink ref="E345" r:id="rId639" xr:uid="{00000000-0004-0000-0000-000039040000}"/>
-    <hyperlink ref="F345" r:id="rId640" xr:uid="{00000000-0004-0000-0000-00003A040000}"/>
-    <hyperlink ref="E346" r:id="rId641" xr:uid="{00000000-0004-0000-0000-00003B040000}"/>
-    <hyperlink ref="F346" r:id="rId642" xr:uid="{00000000-0004-0000-0000-00003C040000}"/>
-    <hyperlink ref="E347" r:id="rId643" xr:uid="{00000000-0004-0000-0000-00003D040000}"/>
-    <hyperlink ref="F348" r:id="rId644" xr:uid="{00000000-0004-0000-0000-00003E040000}"/>
-    <hyperlink ref="E349" r:id="rId645" xr:uid="{00000000-0004-0000-0000-00003F040000}"/>
-    <hyperlink ref="F349" r:id="rId646" xr:uid="{00000000-0004-0000-0000-000040040000}"/>
-    <hyperlink ref="E350" r:id="rId647" xr:uid="{00000000-0004-0000-0000-000041040000}"/>
-    <hyperlink ref="F350" r:id="rId648" xr:uid="{00000000-0004-0000-0000-000042040000}"/>
-    <hyperlink ref="E351" r:id="rId649" xr:uid="{00000000-0004-0000-0000-000043040000}"/>
-    <hyperlink ref="E352" r:id="rId650" xr:uid="{00000000-0004-0000-0000-000045040000}"/>
-    <hyperlink ref="F352" r:id="rId651" xr:uid="{00000000-0004-0000-0000-000046040000}"/>
-    <hyperlink ref="E353" r:id="rId652" xr:uid="{00000000-0004-0000-0000-000047040000}"/>
-    <hyperlink ref="E354" r:id="rId653" xr:uid="{00000000-0004-0000-0000-000049040000}"/>
-    <hyperlink ref="F354" r:id="rId654" xr:uid="{00000000-0004-0000-0000-00004A040000}"/>
-    <hyperlink ref="E355" r:id="rId655" xr:uid="{00000000-0004-0000-0000-00004C040000}"/>
-    <hyperlink ref="E356" r:id="rId656" xr:uid="{00000000-0004-0000-0000-00004D040000}"/>
-    <hyperlink ref="E357" r:id="rId657" xr:uid="{00000000-0004-0000-0000-00004F040000}"/>
-    <hyperlink ref="F357" r:id="rId658" xr:uid="{00000000-0004-0000-0000-000050040000}"/>
-    <hyperlink ref="E358" r:id="rId659" xr:uid="{00000000-0004-0000-0000-000052040000}"/>
-    <hyperlink ref="F358" r:id="rId660" xr:uid="{00000000-0004-0000-0000-000053040000}"/>
-    <hyperlink ref="E359" r:id="rId661" xr:uid="{00000000-0004-0000-0000-000056040000}"/>
-    <hyperlink ref="F359" r:id="rId662" xr:uid="{00000000-0004-0000-0000-000057040000}"/>
-    <hyperlink ref="E360" r:id="rId663" xr:uid="{00000000-0004-0000-0000-000058040000}"/>
-    <hyperlink ref="F360" r:id="rId664" xr:uid="{00000000-0004-0000-0000-000059040000}"/>
-    <hyperlink ref="E361" r:id="rId665" xr:uid="{00000000-0004-0000-0000-00005B040000}"/>
-    <hyperlink ref="E362" r:id="rId666" xr:uid="{00000000-0004-0000-0000-00005C040000}"/>
-    <hyperlink ref="E363" r:id="rId667" xr:uid="{00000000-0004-0000-0000-00005F040000}"/>
-    <hyperlink ref="F363" r:id="rId668" xr:uid="{00000000-0004-0000-0000-000060040000}"/>
-    <hyperlink ref="E364" r:id="rId669" xr:uid="{00000000-0004-0000-0000-000061040000}"/>
-    <hyperlink ref="F364" r:id="rId670" xr:uid="{00000000-0004-0000-0000-000062040000}"/>
-    <hyperlink ref="E365" r:id="rId671" xr:uid="{00000000-0004-0000-0000-000063040000}"/>
-    <hyperlink ref="F365" r:id="rId672" xr:uid="{00000000-0004-0000-0000-000064040000}"/>
-    <hyperlink ref="E366" r:id="rId673" xr:uid="{00000000-0004-0000-0000-000065040000}"/>
-    <hyperlink ref="F366" r:id="rId674" xr:uid="{00000000-0004-0000-0000-000066040000}"/>
-    <hyperlink ref="E367" r:id="rId675" xr:uid="{00000000-0004-0000-0000-000067040000}"/>
-    <hyperlink ref="F367" r:id="rId676" xr:uid="{00000000-0004-0000-0000-000068040000}"/>
-    <hyperlink ref="E368" r:id="rId677" xr:uid="{00000000-0004-0000-0000-000069040000}"/>
-    <hyperlink ref="F368" r:id="rId678" xr:uid="{00000000-0004-0000-0000-00006A040000}"/>
-    <hyperlink ref="E369" r:id="rId679" xr:uid="{00000000-0004-0000-0000-00006B040000}"/>
-    <hyperlink ref="F370" r:id="rId680" xr:uid="{00000000-0004-0000-0000-00006D040000}"/>
-    <hyperlink ref="G370" r:id="rId681" xr:uid="{00000000-0004-0000-0000-00006E040000}"/>
-    <hyperlink ref="E371" r:id="rId682" xr:uid="{00000000-0004-0000-0000-000078040000}"/>
-    <hyperlink ref="F371" r:id="rId683" xr:uid="{00000000-0004-0000-0000-000079040000}"/>
-    <hyperlink ref="E372" r:id="rId684" xr:uid="{00000000-0004-0000-0000-00007A040000}"/>
-    <hyperlink ref="E373" r:id="rId685" xr:uid="{00000000-0004-0000-0000-00007D040000}"/>
-    <hyperlink ref="E374" r:id="rId686" xr:uid="{00000000-0004-0000-0000-00007F040000}"/>
-    <hyperlink ref="F374" r:id="rId687" xr:uid="{00000000-0004-0000-0000-000080040000}"/>
-    <hyperlink ref="G374" r:id="rId688" xr:uid="{00000000-0004-0000-0000-000081040000}"/>
-    <hyperlink ref="E375" r:id="rId689" xr:uid="{00000000-0004-0000-0000-000083040000}"/>
-    <hyperlink ref="E376" r:id="rId690" xr:uid="{00000000-0004-0000-0000-000084040000}"/>
-    <hyperlink ref="E377" r:id="rId691" xr:uid="{00000000-0004-0000-0000-000085040000}"/>
-    <hyperlink ref="F377" r:id="rId692" xr:uid="{00000000-0004-0000-0000-000086040000}"/>
-    <hyperlink ref="G377" r:id="rId693" xr:uid="{00000000-0004-0000-0000-000087040000}"/>
-    <hyperlink ref="E378" r:id="rId694" xr:uid="{00000000-0004-0000-0000-000094040000}"/>
-    <hyperlink ref="F378" r:id="rId695" xr:uid="{00000000-0004-0000-0000-000096040000}"/>
-    <hyperlink ref="E379" r:id="rId696" xr:uid="{00000000-0004-0000-0000-00009C040000}"/>
-    <hyperlink ref="F379" r:id="rId697" xr:uid="{00000000-0004-0000-0000-00009D040000}"/>
-    <hyperlink ref="E380" r:id="rId698" xr:uid="{00000000-0004-0000-0000-00009F040000}"/>
-    <hyperlink ref="F380" r:id="rId699" xr:uid="{00000000-0004-0000-0000-0000A0040000}"/>
-    <hyperlink ref="E381" r:id="rId700" xr:uid="{00000000-0004-0000-0000-0000A1040000}"/>
-    <hyperlink ref="F381" r:id="rId701" xr:uid="{00000000-0004-0000-0000-0000A2040000}"/>
-    <hyperlink ref="E382" r:id="rId702" xr:uid="{00000000-0004-0000-0000-0000A5040000}"/>
-    <hyperlink ref="F382" r:id="rId703" xr:uid="{00000000-0004-0000-0000-0000A6040000}"/>
-    <hyperlink ref="G382" r:id="rId704" xr:uid="{00000000-0004-0000-0000-0000A7040000}"/>
-    <hyperlink ref="E383" r:id="rId705" xr:uid="{00000000-0004-0000-0000-0000A8040000}"/>
-    <hyperlink ref="E384" r:id="rId706" xr:uid="{00000000-0004-0000-0000-0000AD040000}"/>
-    <hyperlink ref="E385" r:id="rId707" xr:uid="{00000000-0004-0000-0000-0000AE040000}"/>
-    <hyperlink ref="E386" r:id="rId708" xr:uid="{00000000-0004-0000-0000-0000B0040000}"/>
-    <hyperlink ref="F386" r:id="rId709" xr:uid="{00000000-0004-0000-0000-0000B1040000}"/>
-    <hyperlink ref="E387" r:id="rId710" xr:uid="{00000000-0004-0000-0000-0000B2040000}"/>
-    <hyperlink ref="F387" r:id="rId711" xr:uid="{00000000-0004-0000-0000-0000B3040000}"/>
-    <hyperlink ref="E388" r:id="rId712" xr:uid="{00000000-0004-0000-0000-0000B5040000}"/>
-    <hyperlink ref="F388" r:id="rId713" xr:uid="{00000000-0004-0000-0000-0000B6040000}"/>
-    <hyperlink ref="E389" r:id="rId714" xr:uid="{00000000-0004-0000-0000-0000B7040000}"/>
-    <hyperlink ref="F389" r:id="rId715" xr:uid="{00000000-0004-0000-0000-0000B8040000}"/>
-    <hyperlink ref="E390" r:id="rId716" xr:uid="{00000000-0004-0000-0000-0000BA040000}"/>
-    <hyperlink ref="F390" r:id="rId717" xr:uid="{00000000-0004-0000-0000-0000BB040000}"/>
-    <hyperlink ref="G390" r:id="rId718" xr:uid="{00000000-0004-0000-0000-0000BC040000}"/>
-    <hyperlink ref="E391" r:id="rId719" xr:uid="{00000000-0004-0000-0000-0000BE040000}"/>
-    <hyperlink ref="F391" r:id="rId720" xr:uid="{00000000-0004-0000-0000-0000BF040000}"/>
-    <hyperlink ref="G391" r:id="rId721" xr:uid="{00000000-0004-0000-0000-0000C0040000}"/>
-    <hyperlink ref="E392" r:id="rId722" xr:uid="{00000000-0004-0000-0000-0000C2040000}"/>
-    <hyperlink ref="F392" r:id="rId723" xr:uid="{00000000-0004-0000-0000-0000C3040000}"/>
-    <hyperlink ref="E393" r:id="rId724" xr:uid="{00000000-0004-0000-0000-0000C4040000}"/>
-    <hyperlink ref="E394" r:id="rId725" xr:uid="{00000000-0004-0000-0000-0000C5040000}"/>
-    <hyperlink ref="E395" r:id="rId726" xr:uid="{00000000-0004-0000-0000-0000C6040000}"/>
-    <hyperlink ref="F395" r:id="rId727" xr:uid="{00000000-0004-0000-0000-0000C7040000}"/>
-    <hyperlink ref="E396" r:id="rId728" xr:uid="{00000000-0004-0000-0000-0000CA040000}"/>
-    <hyperlink ref="E397" r:id="rId729" xr:uid="{00000000-0004-0000-0000-0000CB040000}"/>
-    <hyperlink ref="F397" r:id="rId730" xr:uid="{00000000-0004-0000-0000-0000CC040000}"/>
-    <hyperlink ref="G397" r:id="rId731" xr:uid="{00000000-0004-0000-0000-0000CD040000}"/>
-    <hyperlink ref="E398" r:id="rId732" xr:uid="{00000000-0004-0000-0000-0000D0040000}"/>
-    <hyperlink ref="F398" r:id="rId733" xr:uid="{00000000-0004-0000-0000-0000D1040000}"/>
-    <hyperlink ref="E399" r:id="rId734" xr:uid="{00000000-0004-0000-0000-0000D2040000}"/>
-    <hyperlink ref="E400" r:id="rId735" xr:uid="{00000000-0004-0000-0000-0000D3040000}"/>
-    <hyperlink ref="E401" r:id="rId736" xr:uid="{00000000-0004-0000-0000-0000D4040000}"/>
-    <hyperlink ref="E402" r:id="rId737" xr:uid="{00000000-0004-0000-0000-0000D7040000}"/>
-    <hyperlink ref="E403" r:id="rId738" xr:uid="{00000000-0004-0000-0000-0000D8040000}"/>
-    <hyperlink ref="F403" r:id="rId739" xr:uid="{00000000-0004-0000-0000-0000D9040000}"/>
-    <hyperlink ref="E404" r:id="rId740" xr:uid="{00000000-0004-0000-0000-0000DA040000}"/>
-    <hyperlink ref="F404" r:id="rId741" xr:uid="{00000000-0004-0000-0000-0000DB040000}"/>
-    <hyperlink ref="E405" r:id="rId742" xr:uid="{00000000-0004-0000-0000-0000DC040000}"/>
-    <hyperlink ref="E406" r:id="rId743" xr:uid="{00000000-0004-0000-0000-0000DF040000}"/>
-    <hyperlink ref="F406" r:id="rId744" xr:uid="{00000000-0004-0000-0000-0000E0040000}"/>
-    <hyperlink ref="E273" r:id="rId745" xr:uid="{1F39B638-8349-884B-ABD9-2DFC41CAE56F}"/>
-    <hyperlink ref="E407" r:id="rId746" xr:uid="{EDA42C0A-2150-844A-93D6-7BD8E1CA0B4A}"/>
+    <hyperlink ref="F216" r:id="rId407" xr:uid="{00000000-0004-0000-0000-0000C7020000}"/>
+    <hyperlink ref="E217" r:id="rId408" xr:uid="{00000000-0004-0000-0000-0000C8020000}"/>
+    <hyperlink ref="F217" r:id="rId409" xr:uid="{00000000-0004-0000-0000-0000C9020000}"/>
+    <hyperlink ref="G217" r:id="rId410" xr:uid="{00000000-0004-0000-0000-0000CA020000}"/>
+    <hyperlink ref="E218" r:id="rId411" xr:uid="{00000000-0004-0000-0000-0000CB020000}"/>
+    <hyperlink ref="E219" r:id="rId412" xr:uid="{00000000-0004-0000-0000-0000CC020000}"/>
+    <hyperlink ref="F219" r:id="rId413" xr:uid="{00000000-0004-0000-0000-0000CD020000}"/>
+    <hyperlink ref="E220" r:id="rId414" xr:uid="{00000000-0004-0000-0000-0000CE020000}"/>
+    <hyperlink ref="F220" r:id="rId415" xr:uid="{00000000-0004-0000-0000-0000CF020000}"/>
+    <hyperlink ref="E221" r:id="rId416" xr:uid="{00000000-0004-0000-0000-0000D1020000}"/>
+    <hyperlink ref="F221" r:id="rId417" xr:uid="{00000000-0004-0000-0000-0000D2020000}"/>
+    <hyperlink ref="E222" r:id="rId418" xr:uid="{00000000-0004-0000-0000-0000D3020000}"/>
+    <hyperlink ref="E223" r:id="rId419" xr:uid="{00000000-0004-0000-0000-0000D5020000}"/>
+    <hyperlink ref="F223" r:id="rId420" xr:uid="{00000000-0004-0000-0000-0000D6020000}"/>
+    <hyperlink ref="E224" r:id="rId421" xr:uid="{00000000-0004-0000-0000-0000D9020000}"/>
+    <hyperlink ref="F224" r:id="rId422" xr:uid="{00000000-0004-0000-0000-0000DA020000}"/>
+    <hyperlink ref="G224" r:id="rId423" xr:uid="{00000000-0004-0000-0000-0000DB020000}"/>
+    <hyperlink ref="E225" r:id="rId424" xr:uid="{00000000-0004-0000-0000-0000DC020000}"/>
+    <hyperlink ref="F225" r:id="rId425" xr:uid="{00000000-0004-0000-0000-0000DD020000}"/>
+    <hyperlink ref="G225" r:id="rId426" xr:uid="{00000000-0004-0000-0000-0000DE020000}"/>
+    <hyperlink ref="E226" r:id="rId427" xr:uid="{00000000-0004-0000-0000-0000E0020000}"/>
+    <hyperlink ref="F226" r:id="rId428" xr:uid="{00000000-0004-0000-0000-0000E1020000}"/>
+    <hyperlink ref="E227" r:id="rId429" xr:uid="{00000000-0004-0000-0000-0000E3020000}"/>
+    <hyperlink ref="F227" r:id="rId430" xr:uid="{00000000-0004-0000-0000-0000E4020000}"/>
+    <hyperlink ref="E228" r:id="rId431" xr:uid="{00000000-0004-0000-0000-0000E6020000}"/>
+    <hyperlink ref="E229" r:id="rId432" xr:uid="{00000000-0004-0000-0000-0000E7020000}"/>
+    <hyperlink ref="E230" r:id="rId433" xr:uid="{00000000-0004-0000-0000-0000E8020000}"/>
+    <hyperlink ref="E231" r:id="rId434" xr:uid="{00000000-0004-0000-0000-0000E9020000}"/>
+    <hyperlink ref="F231" r:id="rId435" xr:uid="{00000000-0004-0000-0000-0000EA020000}"/>
+    <hyperlink ref="E232" r:id="rId436" xr:uid="{00000000-0004-0000-0000-0000EB020000}"/>
+    <hyperlink ref="F232" r:id="rId437" xr:uid="{00000000-0004-0000-0000-0000EC020000}"/>
+    <hyperlink ref="E233" r:id="rId438" xr:uid="{00000000-0004-0000-0000-0000EF020000}"/>
+    <hyperlink ref="F233" r:id="rId439" xr:uid="{00000000-0004-0000-0000-0000F0020000}"/>
+    <hyperlink ref="E234" r:id="rId440" xr:uid="{00000000-0004-0000-0000-0000F1020000}"/>
+    <hyperlink ref="F234" r:id="rId441" xr:uid="{00000000-0004-0000-0000-0000F2020000}"/>
+    <hyperlink ref="G234" r:id="rId442" xr:uid="{00000000-0004-0000-0000-0000F3020000}"/>
+    <hyperlink ref="E235" r:id="rId443" xr:uid="{00000000-0004-0000-0000-0000F4020000}"/>
+    <hyperlink ref="F235" r:id="rId444" xr:uid="{00000000-0004-0000-0000-0000F5020000}"/>
+    <hyperlink ref="E236" r:id="rId445" xr:uid="{00000000-0004-0000-0000-0000F8020000}"/>
+    <hyperlink ref="F236" r:id="rId446" xr:uid="{00000000-0004-0000-0000-0000F9020000}"/>
+    <hyperlink ref="G236" r:id="rId447" xr:uid="{00000000-0004-0000-0000-0000FA020000}"/>
+    <hyperlink ref="E237" r:id="rId448" xr:uid="{00000000-0004-0000-0000-0000FE020000}"/>
+    <hyperlink ref="F237" r:id="rId449" xr:uid="{00000000-0004-0000-0000-0000FF020000}"/>
+    <hyperlink ref="G237" r:id="rId450" xr:uid="{00000000-0004-0000-0000-000000030000}"/>
+    <hyperlink ref="E238" r:id="rId451" xr:uid="{00000000-0004-0000-0000-000001030000}"/>
+    <hyperlink ref="F238" r:id="rId452" xr:uid="{00000000-0004-0000-0000-000002030000}"/>
+    <hyperlink ref="G238" r:id="rId453" xr:uid="{00000000-0004-0000-0000-000003030000}"/>
+    <hyperlink ref="E239" r:id="rId454" display="https://github.com/NRCan/PlotFTIR" xr:uid="{00000000-0004-0000-0000-000006030000}"/>
+    <hyperlink ref="E240" r:id="rId455" xr:uid="{00000000-0004-0000-0000-00000B030000}"/>
+    <hyperlink ref="F240" r:id="rId456" xr:uid="{00000000-0004-0000-0000-00000C030000}"/>
+    <hyperlink ref="E241" r:id="rId457" xr:uid="{00000000-0004-0000-0000-00000D030000}"/>
+    <hyperlink ref="E242" r:id="rId458" xr:uid="{00000000-0004-0000-0000-00000F030000}"/>
+    <hyperlink ref="F242" r:id="rId459" xr:uid="{00000000-0004-0000-0000-000010030000}"/>
+    <hyperlink ref="G242" r:id="rId460" xr:uid="{00000000-0004-0000-0000-000011030000}"/>
+    <hyperlink ref="E243" r:id="rId461" xr:uid="{00000000-0004-0000-0000-000012030000}"/>
+    <hyperlink ref="F243" r:id="rId462" xr:uid="{00000000-0004-0000-0000-000013030000}"/>
+    <hyperlink ref="G243" r:id="rId463" xr:uid="{00000000-0004-0000-0000-000014030000}"/>
+    <hyperlink ref="E244" r:id="rId464" xr:uid="{00000000-0004-0000-0000-00001E030000}"/>
+    <hyperlink ref="E245" r:id="rId465" xr:uid="{00000000-0004-0000-0000-00001F030000}"/>
+    <hyperlink ref="F245" r:id="rId466" xr:uid="{00000000-0004-0000-0000-000020030000}"/>
+    <hyperlink ref="E246" r:id="rId467" xr:uid="{00000000-0004-0000-0000-000022030000}"/>
+    <hyperlink ref="E247" r:id="rId468" xr:uid="{00000000-0004-0000-0000-000025030000}"/>
+    <hyperlink ref="E248" r:id="rId469" xr:uid="{00000000-0004-0000-0000-000026030000}"/>
+    <hyperlink ref="E249" r:id="rId470" xr:uid="{00000000-0004-0000-0000-000027030000}"/>
+    <hyperlink ref="F249" r:id="rId471" xr:uid="{00000000-0004-0000-0000-000028030000}"/>
+    <hyperlink ref="E250" r:id="rId472" xr:uid="{00000000-0004-0000-0000-00002C030000}"/>
+    <hyperlink ref="F250" r:id="rId473" xr:uid="{00000000-0004-0000-0000-00002D030000}"/>
+    <hyperlink ref="E251" r:id="rId474" xr:uid="{00000000-0004-0000-0000-000030030000}"/>
+    <hyperlink ref="F251" r:id="rId475" xr:uid="{00000000-0004-0000-0000-000031030000}"/>
+    <hyperlink ref="E252" r:id="rId476" xr:uid="{00000000-0004-0000-0000-000034030000}"/>
+    <hyperlink ref="F252" r:id="rId477" xr:uid="{00000000-0004-0000-0000-000035030000}"/>
+    <hyperlink ref="E253" r:id="rId478" xr:uid="{00000000-0004-0000-0000-000036030000}"/>
+    <hyperlink ref="F253" r:id="rId479" xr:uid="{00000000-0004-0000-0000-000037030000}"/>
+    <hyperlink ref="G253" r:id="rId480" xr:uid="{00000000-0004-0000-0000-000038030000}"/>
+    <hyperlink ref="E254" r:id="rId481" xr:uid="{00000000-0004-0000-0000-00003B030000}"/>
+    <hyperlink ref="E255" r:id="rId482" xr:uid="{00000000-0004-0000-0000-00003C030000}"/>
+    <hyperlink ref="E256" r:id="rId483" xr:uid="{00000000-0004-0000-0000-00003D030000}"/>
+    <hyperlink ref="E257" r:id="rId484" xr:uid="{00000000-0004-0000-0000-000042030000}"/>
+    <hyperlink ref="F257" r:id="rId485" xr:uid="{00000000-0004-0000-0000-000043030000}"/>
+    <hyperlink ref="E258" r:id="rId486" xr:uid="{00000000-0004-0000-0000-000044030000}"/>
+    <hyperlink ref="F258" r:id="rId487" xr:uid="{00000000-0004-0000-0000-000045030000}"/>
+    <hyperlink ref="E259" r:id="rId488" xr:uid="{00000000-0004-0000-0000-00004B030000}"/>
+    <hyperlink ref="E260" r:id="rId489" xr:uid="{00000000-0004-0000-0000-00004C030000}"/>
+    <hyperlink ref="E261" r:id="rId490" xr:uid="{00000000-0004-0000-0000-00004D030000}"/>
+    <hyperlink ref="E262" r:id="rId491" xr:uid="{00000000-0004-0000-0000-000053030000}"/>
+    <hyperlink ref="F262" r:id="rId492" xr:uid="{00000000-0004-0000-0000-000054030000}"/>
+    <hyperlink ref="E263" r:id="rId493" xr:uid="{00000000-0004-0000-0000-000055030000}"/>
+    <hyperlink ref="E264" r:id="rId494" xr:uid="{00000000-0004-0000-0000-000056030000}"/>
+    <hyperlink ref="E265" r:id="rId495" xr:uid="{00000000-0004-0000-0000-000059030000}"/>
+    <hyperlink ref="F265" r:id="rId496" xr:uid="{00000000-0004-0000-0000-00005A030000}"/>
+    <hyperlink ref="E266" r:id="rId497" xr:uid="{00000000-0004-0000-0000-00005B030000}"/>
+    <hyperlink ref="F266" r:id="rId498" xr:uid="{00000000-0004-0000-0000-00005C030000}"/>
+    <hyperlink ref="E267" r:id="rId499" xr:uid="{00000000-0004-0000-0000-00005E030000}"/>
+    <hyperlink ref="F267" r:id="rId500" xr:uid="{00000000-0004-0000-0000-00005F030000}"/>
+    <hyperlink ref="E268" r:id="rId501" xr:uid="{00000000-0004-0000-0000-000060030000}"/>
+    <hyperlink ref="F268" r:id="rId502" xr:uid="{00000000-0004-0000-0000-000061030000}"/>
+    <hyperlink ref="E269" r:id="rId503" xr:uid="{00000000-0004-0000-0000-000062030000}"/>
+    <hyperlink ref="F269" r:id="rId504" xr:uid="{00000000-0004-0000-0000-000063030000}"/>
+    <hyperlink ref="E270" r:id="rId505" xr:uid="{00000000-0004-0000-0000-000064030000}"/>
+    <hyperlink ref="F270" r:id="rId506" xr:uid="{00000000-0004-0000-0000-000065030000}"/>
+    <hyperlink ref="E271" r:id="rId507" xr:uid="{00000000-0004-0000-0000-000067030000}"/>
+    <hyperlink ref="E272" r:id="rId508" xr:uid="{00000000-0004-0000-0000-00006B030000}"/>
+    <hyperlink ref="F272" r:id="rId509" xr:uid="{00000000-0004-0000-0000-00006C030000}"/>
+    <hyperlink ref="E274" r:id="rId510" xr:uid="{00000000-0004-0000-0000-00006E030000}"/>
+    <hyperlink ref="F274" r:id="rId511" xr:uid="{00000000-0004-0000-0000-00006F030000}"/>
+    <hyperlink ref="E275" r:id="rId512" xr:uid="{00000000-0004-0000-0000-000072030000}"/>
+    <hyperlink ref="F275" r:id="rId513" xr:uid="{00000000-0004-0000-0000-000073030000}"/>
+    <hyperlink ref="G275" r:id="rId514" location="!divAbstract" xr:uid="{00000000-0004-0000-0000-000074030000}"/>
+    <hyperlink ref="E276" r:id="rId515" xr:uid="{00000000-0004-0000-0000-000077030000}"/>
+    <hyperlink ref="F276" r:id="rId516" xr:uid="{00000000-0004-0000-0000-000078030000}"/>
+    <hyperlink ref="E277" r:id="rId517" xr:uid="{00000000-0004-0000-0000-000084030000}"/>
+    <hyperlink ref="F277" r:id="rId518" xr:uid="{00000000-0004-0000-0000-000085030000}"/>
+    <hyperlink ref="E278" r:id="rId519" xr:uid="{00000000-0004-0000-0000-000086030000}"/>
+    <hyperlink ref="F278" r:id="rId520" xr:uid="{00000000-0004-0000-0000-000087030000}"/>
+    <hyperlink ref="E279" r:id="rId521" xr:uid="{00000000-0004-0000-0000-000089030000}"/>
+    <hyperlink ref="F279" r:id="rId522" xr:uid="{00000000-0004-0000-0000-00008A030000}"/>
+    <hyperlink ref="G279" r:id="rId523" xr:uid="{00000000-0004-0000-0000-00008B030000}"/>
+    <hyperlink ref="E280" r:id="rId524" xr:uid="{00000000-0004-0000-0000-00008C030000}"/>
+    <hyperlink ref="F280" r:id="rId525" xr:uid="{00000000-0004-0000-0000-00008D030000}"/>
+    <hyperlink ref="E281" r:id="rId526" xr:uid="{00000000-0004-0000-0000-000094030000}"/>
+    <hyperlink ref="F281" r:id="rId527" xr:uid="{00000000-0004-0000-0000-000095030000}"/>
+    <hyperlink ref="E282" r:id="rId528" xr:uid="{00000000-0004-0000-0000-000096030000}"/>
+    <hyperlink ref="E283" r:id="rId529" xr:uid="{00000000-0004-0000-0000-000097030000}"/>
+    <hyperlink ref="E284" r:id="rId530" xr:uid="{00000000-0004-0000-0000-000098030000}"/>
+    <hyperlink ref="E285" r:id="rId531" xr:uid="{00000000-0004-0000-0000-00009B030000}"/>
+    <hyperlink ref="F285" r:id="rId532" xr:uid="{00000000-0004-0000-0000-00009C030000}"/>
+    <hyperlink ref="E286" r:id="rId533" xr:uid="{00000000-0004-0000-0000-00009D030000}"/>
+    <hyperlink ref="E287" r:id="rId534" xr:uid="{00000000-0004-0000-0000-00009F030000}"/>
+    <hyperlink ref="F287" r:id="rId535" xr:uid="{00000000-0004-0000-0000-0000A0030000}"/>
+    <hyperlink ref="E288" r:id="rId536" xr:uid="{00000000-0004-0000-0000-0000A1030000}"/>
+    <hyperlink ref="F288" r:id="rId537" xr:uid="{00000000-0004-0000-0000-0000A2030000}"/>
+    <hyperlink ref="E289" r:id="rId538" xr:uid="{00000000-0004-0000-0000-0000A3030000}"/>
+    <hyperlink ref="F289" r:id="rId539" xr:uid="{00000000-0004-0000-0000-0000A4030000}"/>
+    <hyperlink ref="E290" r:id="rId540" xr:uid="{00000000-0004-0000-0000-0000A6030000}"/>
+    <hyperlink ref="F290" r:id="rId541" xr:uid="{00000000-0004-0000-0000-0000A7030000}"/>
+    <hyperlink ref="E291" r:id="rId542" xr:uid="{00000000-0004-0000-0000-0000A8030000}"/>
+    <hyperlink ref="F291" r:id="rId543" xr:uid="{00000000-0004-0000-0000-0000A9030000}"/>
+    <hyperlink ref="E292" r:id="rId544" xr:uid="{00000000-0004-0000-0000-0000AA030000}"/>
+    <hyperlink ref="E293" r:id="rId545" xr:uid="{00000000-0004-0000-0000-0000AB030000}"/>
+    <hyperlink ref="E294" r:id="rId546" xr:uid="{00000000-0004-0000-0000-0000AC030000}"/>
+    <hyperlink ref="E295" r:id="rId547" xr:uid="{00000000-0004-0000-0000-0000AD030000}"/>
+    <hyperlink ref="F295" r:id="rId548" xr:uid="{00000000-0004-0000-0000-0000AE030000}"/>
+    <hyperlink ref="E296" r:id="rId549" xr:uid="{00000000-0004-0000-0000-0000B1030000}"/>
+    <hyperlink ref="F296" r:id="rId550" xr:uid="{00000000-0004-0000-0000-0000B2030000}"/>
+    <hyperlink ref="E297" r:id="rId551" xr:uid="{00000000-0004-0000-0000-0000B3030000}"/>
+    <hyperlink ref="E298" r:id="rId552" xr:uid="{00000000-0004-0000-0000-0000B4030000}"/>
+    <hyperlink ref="E299" r:id="rId553" xr:uid="{00000000-0004-0000-0000-0000B5030000}"/>
+    <hyperlink ref="F299" r:id="rId554" xr:uid="{00000000-0004-0000-0000-0000B6030000}"/>
+    <hyperlink ref="E300" r:id="rId555" xr:uid="{00000000-0004-0000-0000-0000B7030000}"/>
+    <hyperlink ref="E301" r:id="rId556" xr:uid="{00000000-0004-0000-0000-0000B8030000}"/>
+    <hyperlink ref="F301" r:id="rId557" xr:uid="{00000000-0004-0000-0000-0000B9030000}"/>
+    <hyperlink ref="E302" r:id="rId558" xr:uid="{00000000-0004-0000-0000-0000BA030000}"/>
+    <hyperlink ref="F302" r:id="rId559" xr:uid="{00000000-0004-0000-0000-0000BB030000}"/>
+    <hyperlink ref="E303" r:id="rId560" xr:uid="{00000000-0004-0000-0000-0000BC030000}"/>
+    <hyperlink ref="F303" r:id="rId561" xr:uid="{00000000-0004-0000-0000-0000BD030000}"/>
+    <hyperlink ref="E304" r:id="rId562" xr:uid="{00000000-0004-0000-0000-0000BF030000}"/>
+    <hyperlink ref="F304" r:id="rId563" xr:uid="{00000000-0004-0000-0000-0000C0030000}"/>
+    <hyperlink ref="E305" r:id="rId564" xr:uid="{00000000-0004-0000-0000-0000C1030000}"/>
+    <hyperlink ref="F305" r:id="rId565" xr:uid="{00000000-0004-0000-0000-0000C2030000}"/>
+    <hyperlink ref="E306" r:id="rId566" xr:uid="{00000000-0004-0000-0000-0000C4030000}"/>
+    <hyperlink ref="F306" r:id="rId567" xr:uid="{00000000-0004-0000-0000-0000C5030000}"/>
+    <hyperlink ref="E307" r:id="rId568" xr:uid="{00000000-0004-0000-0000-0000C6030000}"/>
+    <hyperlink ref="F307" r:id="rId569" xr:uid="{00000000-0004-0000-0000-0000C7030000}"/>
+    <hyperlink ref="E308" r:id="rId570" xr:uid="{00000000-0004-0000-0000-0000C8030000}"/>
+    <hyperlink ref="F308" r:id="rId571" xr:uid="{00000000-0004-0000-0000-0000C9030000}"/>
+    <hyperlink ref="E309" r:id="rId572" xr:uid="{00000000-0004-0000-0000-0000CA030000}"/>
+    <hyperlink ref="E310" r:id="rId573" xr:uid="{00000000-0004-0000-0000-0000CC030000}"/>
+    <hyperlink ref="F310" r:id="rId574" xr:uid="{00000000-0004-0000-0000-0000CD030000}"/>
+    <hyperlink ref="E311" r:id="rId575" xr:uid="{00000000-0004-0000-0000-0000CF030000}"/>
+    <hyperlink ref="F311" r:id="rId576" xr:uid="{00000000-0004-0000-0000-0000D0030000}"/>
+    <hyperlink ref="G311" r:id="rId577" xr:uid="{00000000-0004-0000-0000-0000D1030000}"/>
+    <hyperlink ref="E312" r:id="rId578" xr:uid="{00000000-0004-0000-0000-0000D2030000}"/>
+    <hyperlink ref="F312" r:id="rId579" xr:uid="{00000000-0004-0000-0000-0000D3030000}"/>
+    <hyperlink ref="E313" r:id="rId580" xr:uid="{00000000-0004-0000-0000-0000D4030000}"/>
+    <hyperlink ref="E314" r:id="rId581" xr:uid="{00000000-0004-0000-0000-0000D5030000}"/>
+    <hyperlink ref="E315" r:id="rId582" xr:uid="{00000000-0004-0000-0000-0000D6030000}"/>
+    <hyperlink ref="F315" r:id="rId583" xr:uid="{00000000-0004-0000-0000-0000D7030000}"/>
+    <hyperlink ref="E316" r:id="rId584" xr:uid="{00000000-0004-0000-0000-0000D8030000}"/>
+    <hyperlink ref="F316" r:id="rId585" xr:uid="{00000000-0004-0000-0000-0000D9030000}"/>
+    <hyperlink ref="F317" r:id="rId586" xr:uid="{00000000-0004-0000-0000-0000DE030000}"/>
+    <hyperlink ref="G317" r:id="rId587" xr:uid="{00000000-0004-0000-0000-0000DF030000}"/>
+    <hyperlink ref="E318" r:id="rId588" xr:uid="{00000000-0004-0000-0000-0000E0030000}"/>
+    <hyperlink ref="F318" r:id="rId589" xr:uid="{00000000-0004-0000-0000-0000E1030000}"/>
+    <hyperlink ref="G318" r:id="rId590" xr:uid="{00000000-0004-0000-0000-0000E2030000}"/>
+    <hyperlink ref="E319" r:id="rId591" xr:uid="{00000000-0004-0000-0000-0000EB030000}"/>
+    <hyperlink ref="F320" r:id="rId592" xr:uid="{00000000-0004-0000-0000-0000EC030000}"/>
+    <hyperlink ref="E321" r:id="rId593" xr:uid="{00000000-0004-0000-0000-0000F9030000}"/>
+    <hyperlink ref="F321" r:id="rId594" xr:uid="{00000000-0004-0000-0000-0000FA030000}"/>
+    <hyperlink ref="E322" r:id="rId595" xr:uid="{00000000-0004-0000-0000-0000FC030000}"/>
+    <hyperlink ref="F322" r:id="rId596" xr:uid="{00000000-0004-0000-0000-0000FD030000}"/>
+    <hyperlink ref="G322" r:id="rId597" xr:uid="{00000000-0004-0000-0000-0000FE030000}"/>
+    <hyperlink ref="E323" r:id="rId598" xr:uid="{00000000-0004-0000-0000-000002040000}"/>
+    <hyperlink ref="E324" r:id="rId599" xr:uid="{00000000-0004-0000-0000-000003040000}"/>
+    <hyperlink ref="E325" r:id="rId600" xr:uid="{00000000-0004-0000-0000-000005040000}"/>
+    <hyperlink ref="F325" r:id="rId601" xr:uid="{00000000-0004-0000-0000-000006040000}"/>
+    <hyperlink ref="E326" r:id="rId602" xr:uid="{00000000-0004-0000-0000-000009040000}"/>
+    <hyperlink ref="F326" r:id="rId603" xr:uid="{00000000-0004-0000-0000-00000A040000}"/>
+    <hyperlink ref="E327" r:id="rId604" xr:uid="{00000000-0004-0000-0000-00000C040000}"/>
+    <hyperlink ref="E328" r:id="rId605" xr:uid="{00000000-0004-0000-0000-00000F040000}"/>
+    <hyperlink ref="F328" r:id="rId606" xr:uid="{00000000-0004-0000-0000-000010040000}"/>
+    <hyperlink ref="G328" r:id="rId607" xr:uid="{00000000-0004-0000-0000-000011040000}"/>
+    <hyperlink ref="E329" r:id="rId608" xr:uid="{00000000-0004-0000-0000-000016040000}"/>
+    <hyperlink ref="E330" r:id="rId609" xr:uid="{00000000-0004-0000-0000-000019040000}"/>
+    <hyperlink ref="F330" r:id="rId610" xr:uid="{00000000-0004-0000-0000-00001A040000}"/>
+    <hyperlink ref="E331" r:id="rId611" xr:uid="{00000000-0004-0000-0000-00001B040000}"/>
+    <hyperlink ref="F331" r:id="rId612" xr:uid="{00000000-0004-0000-0000-00001C040000}"/>
+    <hyperlink ref="E332" r:id="rId613" xr:uid="{00000000-0004-0000-0000-00001D040000}"/>
+    <hyperlink ref="F332" r:id="rId614" xr:uid="{00000000-0004-0000-0000-00001E040000}"/>
+    <hyperlink ref="E333" r:id="rId615" xr:uid="{00000000-0004-0000-0000-000020040000}"/>
+    <hyperlink ref="F333" r:id="rId616" xr:uid="{00000000-0004-0000-0000-000021040000}"/>
+    <hyperlink ref="G333" r:id="rId617" xr:uid="{00000000-0004-0000-0000-000022040000}"/>
+    <hyperlink ref="E334" r:id="rId618" xr:uid="{00000000-0004-0000-0000-000024040000}"/>
+    <hyperlink ref="F334" r:id="rId619" xr:uid="{00000000-0004-0000-0000-000025040000}"/>
+    <hyperlink ref="E335" r:id="rId620" xr:uid="{00000000-0004-0000-0000-000026040000}"/>
+    <hyperlink ref="F335" r:id="rId621" xr:uid="{00000000-0004-0000-0000-000027040000}"/>
+    <hyperlink ref="E336" r:id="rId622" xr:uid="{00000000-0004-0000-0000-000028040000}"/>
+    <hyperlink ref="F336" r:id="rId623" xr:uid="{00000000-0004-0000-0000-000029040000}"/>
+    <hyperlink ref="E337" r:id="rId624" xr:uid="{00000000-0004-0000-0000-00002A040000}"/>
+    <hyperlink ref="F337" r:id="rId625" xr:uid="{00000000-0004-0000-0000-00002B040000}"/>
+    <hyperlink ref="E338" r:id="rId626" xr:uid="{00000000-0004-0000-0000-00002C040000}"/>
+    <hyperlink ref="E339" r:id="rId627" xr:uid="{00000000-0004-0000-0000-00002D040000}"/>
+    <hyperlink ref="F339" r:id="rId628" xr:uid="{00000000-0004-0000-0000-00002E040000}"/>
+    <hyperlink ref="E340" r:id="rId629" xr:uid="{00000000-0004-0000-0000-00002F040000}"/>
+    <hyperlink ref="F340" r:id="rId630" xr:uid="{00000000-0004-0000-0000-000030040000}"/>
+    <hyperlink ref="E341" r:id="rId631" xr:uid="{00000000-0004-0000-0000-000031040000}"/>
+    <hyperlink ref="F341" r:id="rId632" xr:uid="{00000000-0004-0000-0000-000032040000}"/>
+    <hyperlink ref="E342" r:id="rId633" xr:uid="{00000000-0004-0000-0000-000036040000}"/>
+    <hyperlink ref="E343" r:id="rId634" xr:uid="{00000000-0004-0000-0000-000037040000}"/>
+    <hyperlink ref="F343" r:id="rId635" xr:uid="{00000000-0004-0000-0000-000038040000}"/>
+    <hyperlink ref="E344" r:id="rId636" xr:uid="{00000000-0004-0000-0000-000039040000}"/>
+    <hyperlink ref="F344" r:id="rId637" xr:uid="{00000000-0004-0000-0000-00003A040000}"/>
+    <hyperlink ref="E345" r:id="rId638" xr:uid="{00000000-0004-0000-0000-00003B040000}"/>
+    <hyperlink ref="F345" r:id="rId639" xr:uid="{00000000-0004-0000-0000-00003C040000}"/>
+    <hyperlink ref="E346" r:id="rId640" xr:uid="{00000000-0004-0000-0000-00003D040000}"/>
+    <hyperlink ref="F347" r:id="rId641" xr:uid="{00000000-0004-0000-0000-00003E040000}"/>
+    <hyperlink ref="E348" r:id="rId642" xr:uid="{00000000-0004-0000-0000-00003F040000}"/>
+    <hyperlink ref="F348" r:id="rId643" xr:uid="{00000000-0004-0000-0000-000040040000}"/>
+    <hyperlink ref="E349" r:id="rId644" xr:uid="{00000000-0004-0000-0000-000041040000}"/>
+    <hyperlink ref="F349" r:id="rId645" xr:uid="{00000000-0004-0000-0000-000042040000}"/>
+    <hyperlink ref="E350" r:id="rId646" xr:uid="{00000000-0004-0000-0000-000043040000}"/>
+    <hyperlink ref="E351" r:id="rId647" xr:uid="{00000000-0004-0000-0000-000045040000}"/>
+    <hyperlink ref="F351" r:id="rId648" xr:uid="{00000000-0004-0000-0000-000046040000}"/>
+    <hyperlink ref="E352" r:id="rId649" xr:uid="{00000000-0004-0000-0000-000047040000}"/>
+    <hyperlink ref="E353" r:id="rId650" xr:uid="{00000000-0004-0000-0000-000049040000}"/>
+    <hyperlink ref="F353" r:id="rId651" xr:uid="{00000000-0004-0000-0000-00004A040000}"/>
+    <hyperlink ref="E354" r:id="rId652" xr:uid="{00000000-0004-0000-0000-00004C040000}"/>
+    <hyperlink ref="E355" r:id="rId653" xr:uid="{00000000-0004-0000-0000-00004D040000}"/>
+    <hyperlink ref="E356" r:id="rId654" xr:uid="{00000000-0004-0000-0000-00004F040000}"/>
+    <hyperlink ref="F356" r:id="rId655" xr:uid="{00000000-0004-0000-0000-000050040000}"/>
+    <hyperlink ref="E357" r:id="rId656" xr:uid="{00000000-0004-0000-0000-000052040000}"/>
+    <hyperlink ref="F357" r:id="rId657" xr:uid="{00000000-0004-0000-0000-000053040000}"/>
+    <hyperlink ref="E358" r:id="rId658" xr:uid="{00000000-0004-0000-0000-000056040000}"/>
+    <hyperlink ref="F358" r:id="rId659" xr:uid="{00000000-0004-0000-0000-000057040000}"/>
+    <hyperlink ref="E359" r:id="rId660" xr:uid="{00000000-0004-0000-0000-000058040000}"/>
+    <hyperlink ref="F359" r:id="rId661" xr:uid="{00000000-0004-0000-0000-000059040000}"/>
+    <hyperlink ref="E360" r:id="rId662" xr:uid="{00000000-0004-0000-0000-00005B040000}"/>
+    <hyperlink ref="E361" r:id="rId663" xr:uid="{00000000-0004-0000-0000-00005C040000}"/>
+    <hyperlink ref="E362" r:id="rId664" xr:uid="{00000000-0004-0000-0000-00005F040000}"/>
+    <hyperlink ref="F362" r:id="rId665" xr:uid="{00000000-0004-0000-0000-000060040000}"/>
+    <hyperlink ref="E363" r:id="rId666" xr:uid="{00000000-0004-0000-0000-000061040000}"/>
+    <hyperlink ref="F363" r:id="rId667" xr:uid="{00000000-0004-0000-0000-000062040000}"/>
+    <hyperlink ref="E364" r:id="rId668" xr:uid="{00000000-0004-0000-0000-000063040000}"/>
+    <hyperlink ref="F364" r:id="rId669" xr:uid="{00000000-0004-0000-0000-000064040000}"/>
+    <hyperlink ref="E365" r:id="rId670" xr:uid="{00000000-0004-0000-0000-000065040000}"/>
+    <hyperlink ref="F365" r:id="rId671" xr:uid="{00000000-0004-0000-0000-000066040000}"/>
+    <hyperlink ref="E366" r:id="rId672" xr:uid="{00000000-0004-0000-0000-000067040000}"/>
+    <hyperlink ref="F366" r:id="rId673" xr:uid="{00000000-0004-0000-0000-000068040000}"/>
+    <hyperlink ref="E367" r:id="rId674" xr:uid="{00000000-0004-0000-0000-000069040000}"/>
+    <hyperlink ref="F367" r:id="rId675" xr:uid="{00000000-0004-0000-0000-00006A040000}"/>
+    <hyperlink ref="E368" r:id="rId676" xr:uid="{00000000-0004-0000-0000-00006B040000}"/>
+    <hyperlink ref="F369" r:id="rId677" xr:uid="{00000000-0004-0000-0000-00006D040000}"/>
+    <hyperlink ref="G369" r:id="rId678" xr:uid="{00000000-0004-0000-0000-00006E040000}"/>
+    <hyperlink ref="E370" r:id="rId679" xr:uid="{00000000-0004-0000-0000-000078040000}"/>
+    <hyperlink ref="F370" r:id="rId680" xr:uid="{00000000-0004-0000-0000-000079040000}"/>
+    <hyperlink ref="E371" r:id="rId681" xr:uid="{00000000-0004-0000-0000-00007A040000}"/>
+    <hyperlink ref="E372" r:id="rId682" xr:uid="{00000000-0004-0000-0000-00007D040000}"/>
+    <hyperlink ref="E373" r:id="rId683" xr:uid="{00000000-0004-0000-0000-00007F040000}"/>
+    <hyperlink ref="F373" r:id="rId684" xr:uid="{00000000-0004-0000-0000-000080040000}"/>
+    <hyperlink ref="G373" r:id="rId685" xr:uid="{00000000-0004-0000-0000-000081040000}"/>
+    <hyperlink ref="E374" r:id="rId686" xr:uid="{00000000-0004-0000-0000-000083040000}"/>
+    <hyperlink ref="E375" r:id="rId687" xr:uid="{00000000-0004-0000-0000-000084040000}"/>
+    <hyperlink ref="E376" r:id="rId688" xr:uid="{00000000-0004-0000-0000-000085040000}"/>
+    <hyperlink ref="F376" r:id="rId689" xr:uid="{00000000-0004-0000-0000-000086040000}"/>
+    <hyperlink ref="G376" r:id="rId690" xr:uid="{00000000-0004-0000-0000-000087040000}"/>
+    <hyperlink ref="E377" r:id="rId691" xr:uid="{00000000-0004-0000-0000-000094040000}"/>
+    <hyperlink ref="F377" r:id="rId692" xr:uid="{00000000-0004-0000-0000-000096040000}"/>
+    <hyperlink ref="E378" r:id="rId693" xr:uid="{00000000-0004-0000-0000-00009C040000}"/>
+    <hyperlink ref="F378" r:id="rId694" xr:uid="{00000000-0004-0000-0000-00009D040000}"/>
+    <hyperlink ref="E379" r:id="rId695" xr:uid="{00000000-0004-0000-0000-00009F040000}"/>
+    <hyperlink ref="F379" r:id="rId696" xr:uid="{00000000-0004-0000-0000-0000A0040000}"/>
+    <hyperlink ref="E380" r:id="rId697" xr:uid="{00000000-0004-0000-0000-0000A1040000}"/>
+    <hyperlink ref="F380" r:id="rId698" xr:uid="{00000000-0004-0000-0000-0000A2040000}"/>
+    <hyperlink ref="E381" r:id="rId699" xr:uid="{00000000-0004-0000-0000-0000A5040000}"/>
+    <hyperlink ref="F381" r:id="rId700" xr:uid="{00000000-0004-0000-0000-0000A6040000}"/>
+    <hyperlink ref="G381" r:id="rId701" xr:uid="{00000000-0004-0000-0000-0000A7040000}"/>
+    <hyperlink ref="E382" r:id="rId702" xr:uid="{00000000-0004-0000-0000-0000A8040000}"/>
+    <hyperlink ref="E383" r:id="rId703" xr:uid="{00000000-0004-0000-0000-0000AD040000}"/>
+    <hyperlink ref="E384" r:id="rId704" xr:uid="{00000000-0004-0000-0000-0000AE040000}"/>
+    <hyperlink ref="E385" r:id="rId705" xr:uid="{00000000-0004-0000-0000-0000B0040000}"/>
+    <hyperlink ref="F385" r:id="rId706" xr:uid="{00000000-0004-0000-0000-0000B1040000}"/>
+    <hyperlink ref="E386" r:id="rId707" xr:uid="{00000000-0004-0000-0000-0000B2040000}"/>
+    <hyperlink ref="F386" r:id="rId708" xr:uid="{00000000-0004-0000-0000-0000B3040000}"/>
+    <hyperlink ref="E387" r:id="rId709" xr:uid="{00000000-0004-0000-0000-0000B5040000}"/>
+    <hyperlink ref="F387" r:id="rId710" xr:uid="{00000000-0004-0000-0000-0000B6040000}"/>
+    <hyperlink ref="E388" r:id="rId711" xr:uid="{00000000-0004-0000-0000-0000B7040000}"/>
+    <hyperlink ref="F388" r:id="rId712" xr:uid="{00000000-0004-0000-0000-0000B8040000}"/>
+    <hyperlink ref="E389" r:id="rId713" xr:uid="{00000000-0004-0000-0000-0000BA040000}"/>
+    <hyperlink ref="F389" r:id="rId714" xr:uid="{00000000-0004-0000-0000-0000BB040000}"/>
+    <hyperlink ref="G389" r:id="rId715" xr:uid="{00000000-0004-0000-0000-0000BC040000}"/>
+    <hyperlink ref="E390" r:id="rId716" xr:uid="{00000000-0004-0000-0000-0000BE040000}"/>
+    <hyperlink ref="F390" r:id="rId717" xr:uid="{00000000-0004-0000-0000-0000BF040000}"/>
+    <hyperlink ref="G390" r:id="rId718" xr:uid="{00000000-0004-0000-0000-0000C0040000}"/>
+    <hyperlink ref="E391" r:id="rId719" xr:uid="{00000000-0004-0000-0000-0000C2040000}"/>
+    <hyperlink ref="F391" r:id="rId720" xr:uid="{00000000-0004-0000-0000-0000C3040000}"/>
+    <hyperlink ref="E392" r:id="rId721" xr:uid="{00000000-0004-0000-0000-0000C4040000}"/>
+    <hyperlink ref="E393" r:id="rId722" xr:uid="{00000000-0004-0000-0000-0000C5040000}"/>
+    <hyperlink ref="E394" r:id="rId723" xr:uid="{00000000-0004-0000-0000-0000C6040000}"/>
+    <hyperlink ref="F394" r:id="rId724" xr:uid="{00000000-0004-0000-0000-0000C7040000}"/>
+    <hyperlink ref="E395" r:id="rId725" xr:uid="{00000000-0004-0000-0000-0000CA040000}"/>
+    <hyperlink ref="E396" r:id="rId726" xr:uid="{00000000-0004-0000-0000-0000CB040000}"/>
+    <hyperlink ref="F396" r:id="rId727" xr:uid="{00000000-0004-0000-0000-0000CC040000}"/>
+    <hyperlink ref="G396" r:id="rId728" xr:uid="{00000000-0004-0000-0000-0000CD040000}"/>
+    <hyperlink ref="E397" r:id="rId729" xr:uid="{00000000-0004-0000-0000-0000D0040000}"/>
+    <hyperlink ref="F397" r:id="rId730" xr:uid="{00000000-0004-0000-0000-0000D1040000}"/>
+    <hyperlink ref="E398" r:id="rId731" xr:uid="{00000000-0004-0000-0000-0000D2040000}"/>
+    <hyperlink ref="E399" r:id="rId732" xr:uid="{00000000-0004-0000-0000-0000D3040000}"/>
+    <hyperlink ref="E400" r:id="rId733" xr:uid="{00000000-0004-0000-0000-0000D4040000}"/>
+    <hyperlink ref="E401" r:id="rId734" xr:uid="{00000000-0004-0000-0000-0000D7040000}"/>
+    <hyperlink ref="E402" r:id="rId735" xr:uid="{00000000-0004-0000-0000-0000D8040000}"/>
+    <hyperlink ref="F402" r:id="rId736" xr:uid="{00000000-0004-0000-0000-0000D9040000}"/>
+    <hyperlink ref="E403" r:id="rId737" xr:uid="{00000000-0004-0000-0000-0000DA040000}"/>
+    <hyperlink ref="F403" r:id="rId738" xr:uid="{00000000-0004-0000-0000-0000DB040000}"/>
+    <hyperlink ref="E404" r:id="rId739" xr:uid="{00000000-0004-0000-0000-0000DC040000}"/>
+    <hyperlink ref="E405" r:id="rId740" xr:uid="{00000000-0004-0000-0000-0000DF040000}"/>
+    <hyperlink ref="F405" r:id="rId741" xr:uid="{00000000-0004-0000-0000-0000E0040000}"/>
+    <hyperlink ref="E273" r:id="rId742" xr:uid="{1F39B638-8349-884B-ABD9-2DFC41CAE56F}"/>
+    <hyperlink ref="E406" r:id="rId743" xr:uid="{EDA42C0A-2150-844A-93D6-7BD8E1CA0B4A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="80" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>